<commit_message>
Enhance README.md with sponsor details; update sponsor logo handling in app.js and CSS for improved display; complete tasks related to sponsor logos and links in planning documents; increment versioning in index.html, app.js, and service worker for cache updates.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="HH:MM"/>
     <numFmt numFmtId="168" formatCode="YYYY-MM-DD HH:MM"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +41,12 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -81,6 +90,9 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4339,7 +4351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O192"/>
+  <dimension ref="A1:S192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4354,6 +4366,10 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="13"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4432,6 +4448,26 @@
           <t>Примечание (EN)</t>
         </is>
       </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>Сайт</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>Логотип</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>Спонсор (RU)</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>Спонсор (EN)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="43.5" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -4812,6 +4848,26 @@
       <c r="J9" t="n">
         <v>15</v>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>https://gammatech.pro/</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>gammatech.png</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Гамматек</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Gammatech</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="174" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -4857,6 +4913,26 @@
       <c r="J10" t="n">
         <v>15</v>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>https://edigitizer.ru/</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>digitizer.svg</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Диджитайзер</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Digitizer</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="72.5" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -4896,6 +4972,26 @@
       </c>
       <c r="J11" t="n">
         <v>15</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>https://spegroup.ru/</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>spegroup.svg</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Научное оборудование</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Scientific Equipment</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="261" customHeight="1">

</xml_diff>

<commit_message>
Update .gitignore to include new schedule overview PDFs; enhance README.md with updated audience room details and duration settings; modify app.js to support new social venue mapping and improve section sorting logic; increment versioning in index.html, app.js, and sw.js for cache management consistency.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
     <numFmt numFmtId="167" formatCode="HH:MM"/>
     <numFmt numFmtId="168" formatCode="YYYY-MM-DD HH:MM"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -93,6 +94,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2564,6 +2566,11 @@
           <t>Concert</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3497,6 +3504,11 @@
           <t>Boat excursion on the Amur River</t>
         </is>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>причал</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3521,6 +3533,11 @@
       <c r="F63" t="inlineStr">
         <is>
           <t>Conference dinner</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>интурист</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4528,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" ht="29" customHeight="1">
@@ -4556,7 +4573,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" ht="116" customHeight="1">
@@ -14850,7 +14867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14919,6 +14936,21 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>46280.72569444445</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Юбилейные доклады — 30 мин. Концерт в актовом зале. Экскурсия — 4-й причал; банкет — ресторан «Интурист».</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Anniversary talks are 30 min. Concert in the Assembly Hall. Excursion: Pier 4; conference dinner: Restaurant Inturist.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update programme data and regenerate site data.js for NUCLEUS-2026 conference schedule; changes include new session details and updated event timings.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11220" yWindow="3910" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Настройки" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,13 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
-    <numFmt numFmtId="167" formatCode="HH:MM"/>
-    <numFmt numFmtId="168" formatCode="YYYY-MM-DD HH:MM"/>
-    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -43,8 +42,10 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -61,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -89,12 +90,10 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,7 +460,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="3"/>
@@ -694,7 +693,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="3"/>
@@ -1019,7 +1018,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M84"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="3"/>
@@ -1029,7 +1028,6 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="11"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2305,7 +2303,7 @@
       <c r="B31" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="3" t="n">
         <v>0.6458333333333334</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -2486,7 +2484,7 @@
       <c r="B37" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C37" s="3" t="n">
         <v>0.7291666666666666</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -2968,7 +2966,7 @@
       <c r="B49" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C49" s="6" t="n">
+      <c r="C49" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -3906,7 +3904,7 @@
       <c r="B72" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C72" s="6" t="n">
+      <c r="C72" s="3" t="n">
         <v>0.6354166666666666</v>
       </c>
       <c r="D72" t="inlineStr">
@@ -4369,7 +4367,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S192"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -4379,14 +4377,13 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="37.140625" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="13"/>
     <col width="28" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="18" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4465,22 +4462,22 @@
           <t>Примечание (EN)</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Сайт</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Логотип</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>Спонсор (RU)</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>Спонсор (EN)</t>
         </is>
@@ -4531,7 +4528,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" ht="29" customHeight="1">
+    <row r="3" ht="29.1" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>P-J2</t>
@@ -4576,7 +4573,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" ht="116" customHeight="1">
+    <row r="4" ht="116.1" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>P-01</t>
@@ -4721,7 +4718,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="290" customHeight="1">
+    <row r="7" ht="290.1" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>P-04</t>
@@ -4771,7 +4768,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="232" customHeight="1">
+    <row r="8" ht="231.95" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>P-05</t>
@@ -4951,7 +4948,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="72.5" customHeight="1">
+    <row r="11" ht="72.59999999999999" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>P-S3</t>
@@ -5061,7 +5058,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="145" customHeight="1">
+    <row r="13" ht="144.95" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>P-07</t>
@@ -5111,7 +5108,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="145" customHeight="1">
+    <row r="14" ht="144.95" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>P-08</t>
@@ -5161,7 +5158,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="203" customHeight="1">
+    <row r="15" ht="203.1" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>P-09</t>
@@ -5211,7 +5208,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="203" customHeight="1">
+    <row r="16" ht="203.1" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>P-10</t>
@@ -5361,7 +5358,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="232" customHeight="1">
+    <row r="19" ht="231.95" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>P-13</t>
@@ -5461,7 +5458,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="203" customHeight="1">
+    <row r="21" ht="203.1" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>P-15</t>
@@ -5511,7 +5508,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="145" customHeight="1">
+    <row r="22" ht="144.95" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>P-16</t>
@@ -5561,7 +5558,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="101.5" customHeight="1">
+    <row r="23" ht="101.45" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>P-17</t>
@@ -5761,7 +5758,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="145" customHeight="1">
+    <row r="27" ht="144.95" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>P-21</t>
@@ -5811,7 +5808,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="290" customHeight="1">
+    <row r="28" ht="290.1" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>P-22</t>
@@ -5861,7 +5858,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="145" customHeight="1">
+    <row r="29" ht="144.95" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>P-23</t>
@@ -5911,7 +5908,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="72.5" customHeight="1">
+    <row r="30" ht="72.59999999999999" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>P-24</t>
@@ -6006,7 +6003,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="275.5" customHeight="1">
+    <row r="32" ht="275.45" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>P-26</t>
@@ -6106,7 +6103,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="116" customHeight="1">
+    <row r="34" ht="116.1" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>P-28</t>
@@ -6467,7 +6464,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Эстония</t>
+          <t>Garon Sci. Lab., Fonoriton LtD (Tallinn, Estonia)</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -6481,7 +6478,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="116" customHeight="1">
+    <row r="42" ht="116.1" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>S1-04</t>
@@ -6606,7 +6603,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="159.5" customHeight="1">
+    <row r="45" ht="159.6" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
           <t>S1-07</t>
@@ -6696,7 +6693,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="246.5" customHeight="1">
+    <row r="47" ht="246.6" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
           <t>S1-09</t>
@@ -6741,7 +6738,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="377" customHeight="1">
+    <row r="48" ht="377.1" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
           <t>S1-10</t>
@@ -6786,7 +6783,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="159.5" customHeight="1">
+    <row r="49" ht="159.6" customHeight="1">
       <c r="A49" t="inlineStr">
         <is>
           <t>S1-11</t>
@@ -6831,7 +6828,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="159.5" customHeight="1">
+    <row r="50" ht="159.6" customHeight="1">
       <c r="A50" t="inlineStr">
         <is>
           <t>S1-12</t>
@@ -6876,7 +6873,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="72.5" customHeight="1">
+    <row r="51" ht="72.59999999999999" customHeight="1">
       <c r="A51" t="inlineStr">
         <is>
           <t>S1-13</t>
@@ -6961,7 +6958,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="116" customHeight="1">
+    <row r="53" ht="116.1" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
           <t>S1-15</t>
@@ -7046,7 +7043,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="203" customHeight="1">
+    <row r="55" ht="203.1" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
           <t>S1-17</t>
@@ -7091,7 +7088,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="203" customHeight="1">
+    <row r="56" ht="203.1" customHeight="1">
       <c r="A56" t="inlineStr">
         <is>
           <t>S1-18</t>
@@ -7162,7 +7159,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Узбекистан</t>
+          <t>Наманганский государственный технический университет (Наманган, Узбекистан)</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -7176,7 +7173,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="246.5" customHeight="1">
+    <row r="58" ht="246.6" customHeight="1">
       <c r="A58" t="inlineStr">
         <is>
           <t>S1-20</t>
@@ -7261,7 +7258,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="145" customHeight="1">
+    <row r="60" ht="144.95" customHeight="1">
       <c r="A60" t="inlineStr">
         <is>
           <t>S1-22</t>
@@ -7396,7 +7393,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="101.5" customHeight="1">
+    <row r="63" ht="101.45" customHeight="1">
       <c r="A63" t="inlineStr">
         <is>
           <t>S1-25</t>
@@ -7476,7 +7473,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="116" customHeight="1">
+    <row r="65" ht="116.1" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
           <t>S1-27</t>
@@ -7568,7 +7565,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="319" customHeight="1">
+    <row r="67" ht="318.95" customHeight="1">
       <c r="A67" t="inlineStr">
         <is>
           <t>S2-03</t>
@@ -7615,7 +7612,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="290" customHeight="1">
+    <row r="68" ht="290.1" customHeight="1">
       <c r="A68" t="inlineStr">
         <is>
           <t>S2-04</t>
@@ -7662,7 +7659,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="362.5" customHeight="1">
+    <row r="69" ht="362.45" customHeight="1">
       <c r="A69" t="inlineStr">
         <is>
           <t>S2-05</t>
@@ -7704,7 +7701,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="275.5" customHeight="1">
+    <row r="70" ht="275.45" customHeight="1">
       <c r="A70" t="inlineStr">
         <is>
           <t>S2-06</t>
@@ -7751,7 +7748,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="72.5" customHeight="1">
+    <row r="71" ht="72.59999999999999" customHeight="1">
       <c r="A71" t="inlineStr">
         <is>
           <t>S2-07</t>
@@ -7843,7 +7840,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="232" customHeight="1">
+    <row r="73" ht="231.95" customHeight="1">
       <c r="A73" t="inlineStr">
         <is>
           <t>S2-10</t>
@@ -7885,7 +7882,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="203" customHeight="1">
+    <row r="74" ht="203.1" customHeight="1">
       <c r="A74" t="inlineStr">
         <is>
           <t>S2-11</t>
@@ -7932,7 +7929,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="203" customHeight="1">
+    <row r="75" ht="203.1" customHeight="1">
       <c r="A75" t="inlineStr">
         <is>
           <t>S2-12</t>
@@ -7979,7 +7976,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="203" customHeight="1">
+    <row r="76" ht="203.1" customHeight="1">
       <c r="A76" t="inlineStr">
         <is>
           <t>S2-13</t>
@@ -8243,7 +8240,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="290" customHeight="1">
+    <row r="82" ht="290.1" customHeight="1">
       <c r="A82" t="inlineStr">
         <is>
           <t>S2-20</t>
@@ -8288,7 +8285,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="145" customHeight="1">
+    <row r="83" ht="144.95" customHeight="1">
       <c r="A83" t="inlineStr">
         <is>
           <t>S2-21</t>
@@ -8333,7 +8330,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="145" customHeight="1">
+    <row r="84" ht="144.95" customHeight="1">
       <c r="A84" t="inlineStr">
         <is>
           <t>S2-22</t>
@@ -8359,7 +8356,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Бангладеш</t>
+          <t>Department of Physics, Jagannath University (Dhaka, Bangladesh)</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -8415,7 +8412,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="203" customHeight="1">
+    <row r="86" ht="203.1" customHeight="1">
       <c r="A86" t="inlineStr">
         <is>
           <t>S2-24</t>
@@ -8457,7 +8454,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="188.5" customHeight="1">
+    <row r="87" ht="188.45" customHeight="1">
       <c r="A87" t="inlineStr">
         <is>
           <t>S2-25</t>
@@ -8551,7 +8548,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="290" customHeight="1">
+    <row r="89" ht="290.1" customHeight="1">
       <c r="A89" t="inlineStr">
         <is>
           <t>S2-27</t>
@@ -8593,7 +8590,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="159.5" customHeight="1">
+    <row r="90" ht="159.6" customHeight="1">
       <c r="A90" t="inlineStr">
         <is>
           <t>S2-28</t>
@@ -8635,7 +8632,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="145" customHeight="1">
+    <row r="91" ht="144.95" customHeight="1">
       <c r="A91" t="inlineStr">
         <is>
           <t>S2-29</t>
@@ -8717,7 +8714,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="232" customHeight="1">
+    <row r="93" ht="231.95" customHeight="1">
       <c r="A93" t="inlineStr">
         <is>
           <t>S2-31</t>
@@ -8797,7 +8794,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="203" customHeight="1">
+    <row r="95" ht="203.1" customHeight="1">
       <c r="A95" t="inlineStr">
         <is>
           <t>S2-33</t>
@@ -8837,7 +8834,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="145" customHeight="1">
+    <row r="96" ht="144.95" customHeight="1">
       <c r="A96" t="inlineStr">
         <is>
           <t>S2-34</t>
@@ -8877,7 +8874,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="188.5" customHeight="1">
+    <row r="97" ht="188.45" customHeight="1">
       <c r="A97" t="inlineStr">
         <is>
           <t>S2-35</t>
@@ -8922,7 +8919,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="188.5" customHeight="1">
+    <row r="98" ht="188.45" customHeight="1">
       <c r="A98" t="inlineStr">
         <is>
           <t>S2-36</t>
@@ -8967,7 +8964,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="246.5" customHeight="1">
+    <row r="99" ht="246.6" customHeight="1">
       <c r="A99" t="inlineStr">
         <is>
           <t>S3-01</t>
@@ -9012,7 +9009,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="159.5" customHeight="1">
+    <row r="100" ht="159.6" customHeight="1">
       <c r="A100" t="inlineStr">
         <is>
           <t>S3-02</t>
@@ -9057,7 +9054,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="188.5" customHeight="1">
+    <row r="101" ht="188.45" customHeight="1">
       <c r="A101" t="inlineStr">
         <is>
           <t>S3-03</t>
@@ -9102,7 +9099,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="290" customHeight="1">
+    <row r="102" ht="290.1" customHeight="1">
       <c r="A102" t="inlineStr">
         <is>
           <t>S3-04</t>
@@ -9142,7 +9139,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="290" customHeight="1">
+    <row r="103" ht="290.1" customHeight="1">
       <c r="A103" t="inlineStr">
         <is>
           <t>S3-05</t>
@@ -9187,7 +9184,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="232" customHeight="1">
+    <row r="104" ht="231.95" customHeight="1">
       <c r="A104" t="inlineStr">
         <is>
           <t>S3-06</t>
@@ -9227,7 +9224,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="319" customHeight="1">
+    <row r="105" ht="318.95" customHeight="1">
       <c r="A105" t="inlineStr">
         <is>
           <t>S3-07</t>
@@ -9272,7 +9269,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="333.5" customHeight="1">
+    <row r="106" ht="333.6" customHeight="1">
       <c r="A106" t="inlineStr">
         <is>
           <t>S3-08</t>
@@ -9317,7 +9314,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="145" customHeight="1">
+    <row r="107" ht="144.95" customHeight="1">
       <c r="A107" t="inlineStr">
         <is>
           <t>S3-09</t>
@@ -9357,7 +9354,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="246.5" customHeight="1">
+    <row r="108" ht="246.6" customHeight="1">
       <c r="A108" t="inlineStr">
         <is>
           <t>S3-10</t>
@@ -9402,7 +9399,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="145" customHeight="1">
+    <row r="109" ht="144.95" customHeight="1">
       <c r="A109" t="inlineStr">
         <is>
           <t>S3-11</t>
@@ -9447,7 +9444,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="275.5" customHeight="1">
+    <row r="110" ht="275.45" customHeight="1">
       <c r="A110" t="inlineStr">
         <is>
           <t>S3-12</t>
@@ -9487,7 +9484,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="188.5" customHeight="1">
+    <row r="111" ht="188.45" customHeight="1">
       <c r="A111" t="inlineStr">
         <is>
           <t>S3-13</t>
@@ -9532,7 +9529,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="116" customHeight="1">
+    <row r="112" ht="116.1" customHeight="1">
       <c r="A112" t="inlineStr">
         <is>
           <t>S3-14</t>
@@ -9577,7 +9574,7 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="246.5" customHeight="1">
+    <row r="113" ht="246.6" customHeight="1">
       <c r="A113" t="inlineStr">
         <is>
           <t>S3-15</t>
@@ -9617,7 +9614,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="188.5" customHeight="1">
+    <row r="114" ht="188.45" customHeight="1">
       <c r="A114" t="inlineStr">
         <is>
           <t>S3-16</t>
@@ -9662,7 +9659,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="333.5" customHeight="1">
+    <row r="115" ht="333.6" customHeight="1">
       <c r="A115" t="inlineStr">
         <is>
           <t>S3-17</t>
@@ -9702,7 +9699,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="203" customHeight="1">
+    <row r="116" ht="203.1" customHeight="1">
       <c r="A116" t="inlineStr">
         <is>
           <t>S3-18</t>
@@ -9787,7 +9784,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="275.5" customHeight="1">
+    <row r="118" ht="275.45" customHeight="1">
       <c r="A118" t="inlineStr">
         <is>
           <t>S3-20</t>
@@ -9832,7 +9829,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="203" customHeight="1">
+    <row r="119" ht="203.1" customHeight="1">
       <c r="A119" t="inlineStr">
         <is>
           <t>S3-21</t>
@@ -9877,7 +9874,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="203" customHeight="1">
+    <row r="120" ht="203.1" customHeight="1">
       <c r="A120" t="inlineStr">
         <is>
           <t>S3-22</t>
@@ -9957,7 +9954,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="188.5" customHeight="1">
+    <row r="122" ht="188.45" customHeight="1">
       <c r="A122" t="inlineStr">
         <is>
           <t>S3-24</t>
@@ -10132,7 +10129,7 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="362.5" customHeight="1">
+    <row r="126" ht="362.45" customHeight="1">
       <c r="A126" t="inlineStr">
         <is>
           <t>S4-01</t>
@@ -10177,7 +10174,7 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="145" customHeight="1">
+    <row r="127" ht="144.95" customHeight="1">
       <c r="A127" t="inlineStr">
         <is>
           <t>S4-02</t>
@@ -10222,7 +10219,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="290" customHeight="1">
+    <row r="128" ht="290.1" customHeight="1">
       <c r="A128" t="inlineStr">
         <is>
           <t>S4-03</t>
@@ -10307,7 +10304,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="232" customHeight="1">
+    <row r="130" ht="231.95" customHeight="1">
       <c r="A130" t="inlineStr">
         <is>
           <t>S4-05</t>
@@ -10352,7 +10349,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="275.5" customHeight="1">
+    <row r="131" ht="275.45" customHeight="1">
       <c r="A131" t="inlineStr">
         <is>
           <t>S4-06</t>
@@ -10442,7 +10439,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="246.5" customHeight="1">
+    <row r="133" ht="246.6" customHeight="1">
       <c r="A133" t="inlineStr">
         <is>
           <t>S4-08</t>
@@ -10534,7 +10531,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="188.5" customHeight="1">
+    <row r="135" ht="188.45" customHeight="1">
       <c r="A135" t="inlineStr">
         <is>
           <t>S4-11</t>
@@ -10581,7 +10578,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="246.5" customHeight="1">
+    <row r="136" ht="246.6" customHeight="1">
       <c r="A136" t="inlineStr">
         <is>
           <t>S4-12</t>
@@ -10675,7 +10672,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="246.5" customHeight="1">
+    <row r="138" ht="246.6" customHeight="1">
       <c r="A138" t="inlineStr">
         <is>
           <t>S4-15</t>
@@ -10765,7 +10762,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="145" customHeight="1">
+    <row r="140" ht="144.95" customHeight="1">
       <c r="A140" t="inlineStr">
         <is>
           <t>S4-17</t>
@@ -10810,7 +10807,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="145" customHeight="1">
+    <row r="141" ht="144.95" customHeight="1">
       <c r="A141" t="inlineStr">
         <is>
           <t>S4-18</t>
@@ -10895,7 +10892,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="232" customHeight="1">
+    <row r="143" ht="231.95" customHeight="1">
       <c r="A143" t="inlineStr">
         <is>
           <t>S4-20</t>
@@ -10940,7 +10937,7 @@
         </is>
       </c>
     </row>
-    <row r="144" ht="159.5" customHeight="1">
+    <row r="144" ht="159.6" customHeight="1">
       <c r="A144" t="inlineStr">
         <is>
           <t>S4-21</t>
@@ -10985,7 +10982,7 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="246.5" customHeight="1">
+    <row r="145" ht="246.6" customHeight="1">
       <c r="A145" t="inlineStr">
         <is>
           <t>S4-22</t>
@@ -11030,7 +11027,7 @@
         </is>
       </c>
     </row>
-    <row r="146" ht="203" customHeight="1">
+    <row r="146" ht="203.1" customHeight="1">
       <c r="A146" t="inlineStr">
         <is>
           <t>S4-23</t>
@@ -11075,7 +11072,7 @@
         </is>
       </c>
     </row>
-    <row r="147" ht="319" customHeight="1">
+    <row r="147" ht="318.95" customHeight="1">
       <c r="A147" t="inlineStr">
         <is>
           <t>S4-24</t>
@@ -11165,7 +11162,7 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="72.5" customHeight="1">
+    <row r="149" ht="72.59999999999999" customHeight="1">
       <c r="A149" t="inlineStr">
         <is>
           <t>S4-26</t>
@@ -11250,7 +11247,7 @@
         </is>
       </c>
     </row>
-    <row r="151" ht="319" customHeight="1">
+    <row r="151" ht="318.95" customHeight="1">
       <c r="A151" t="inlineStr">
         <is>
           <t>S4-28</t>
@@ -11295,7 +11292,7 @@
         </is>
       </c>
     </row>
-    <row r="152" ht="290" customHeight="1">
+    <row r="152" ht="290.1" customHeight="1">
       <c r="A152" t="inlineStr">
         <is>
           <t>S5-01</t>
@@ -11340,7 +11337,7 @@
         </is>
       </c>
     </row>
-    <row r="153" ht="246.5" customHeight="1">
+    <row r="153" ht="246.6" customHeight="1">
       <c r="A153" t="inlineStr">
         <is>
           <t>S5-02</t>
@@ -11560,7 +11557,7 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="188.5" customHeight="1">
+    <row r="158" ht="188.45" customHeight="1">
       <c r="A158" t="inlineStr">
         <is>
           <t>S5-07</t>
@@ -11695,7 +11692,7 @@
         </is>
       </c>
     </row>
-    <row r="161" ht="246.5" customHeight="1">
+    <row r="161" ht="246.6" customHeight="1">
       <c r="A161" t="inlineStr">
         <is>
           <t>S6-01</t>
@@ -11740,7 +11737,7 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="232" customHeight="1">
+    <row r="162" ht="231.95" customHeight="1">
       <c r="A162" t="inlineStr">
         <is>
           <t>S6-02</t>
@@ -11785,7 +11782,7 @@
         </is>
       </c>
     </row>
-    <row r="163" ht="58" customHeight="1">
+    <row r="163" ht="57.95" customHeight="1">
       <c r="A163" t="inlineStr">
         <is>
           <t>S6-03</t>
@@ -11870,7 +11867,7 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="101.5" customHeight="1">
+    <row r="165" ht="101.45" customHeight="1">
       <c r="A165" t="inlineStr">
         <is>
           <t>S6-05</t>
@@ -11960,7 +11957,7 @@
         </is>
       </c>
     </row>
-    <row r="167" ht="145" customHeight="1">
+    <row r="167" ht="144.95" customHeight="1">
       <c r="A167" t="inlineStr">
         <is>
           <t>S6-07</t>
@@ -11986,7 +11983,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Пакистан</t>
+          <t>Institute of Space Technology (Islamabad, Pakistan)</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -12040,7 +12037,7 @@
         </is>
       </c>
     </row>
-    <row r="169" ht="145" customHeight="1">
+    <row r="169" ht="144.95" customHeight="1">
       <c r="A169" t="inlineStr">
         <is>
           <t>S7-01</t>
@@ -12080,7 +12077,7 @@
         </is>
       </c>
     </row>
-    <row r="170" ht="188.5" customHeight="1">
+    <row r="170" ht="188.45" customHeight="1">
       <c r="A170" t="inlineStr">
         <is>
           <t>S7-02</t>
@@ -12125,7 +12122,7 @@
         </is>
       </c>
     </row>
-    <row r="171" ht="159.5" customHeight="1">
+    <row r="171" ht="159.6" customHeight="1">
       <c r="A171" t="inlineStr">
         <is>
           <t>S7-03</t>
@@ -12170,7 +12167,7 @@
         </is>
       </c>
     </row>
-    <row r="172" ht="203" customHeight="1">
+    <row r="172" ht="203.1" customHeight="1">
       <c r="A172" t="inlineStr">
         <is>
           <t>S7-04</t>
@@ -12215,7 +12212,7 @@
         </is>
       </c>
     </row>
-    <row r="173" ht="159.5" customHeight="1">
+    <row r="173" ht="159.6" customHeight="1">
       <c r="A173" t="inlineStr">
         <is>
           <t>S7-05</t>
@@ -12260,7 +12257,7 @@
         </is>
       </c>
     </row>
-    <row r="174" ht="159.5" customHeight="1">
+    <row r="174" ht="159.6" customHeight="1">
       <c r="A174" t="inlineStr">
         <is>
           <t>S7-06</t>
@@ -12305,7 +12302,7 @@
         </is>
       </c>
     </row>
-    <row r="175" ht="290" customHeight="1">
+    <row r="175" ht="290.1" customHeight="1">
       <c r="A175" t="inlineStr">
         <is>
           <t>S7-07</t>
@@ -12350,7 +12347,7 @@
         </is>
       </c>
     </row>
-    <row r="176" ht="232" customHeight="1">
+    <row r="176" ht="231.95" customHeight="1">
       <c r="A176" t="inlineStr">
         <is>
           <t>S7-08</t>
@@ -12480,7 +12477,7 @@
         </is>
       </c>
     </row>
-    <row r="179" ht="319" customHeight="1">
+    <row r="179" ht="318.95" customHeight="1">
       <c r="A179" t="inlineStr">
         <is>
           <t>S7-11</t>
@@ -12525,7 +12522,7 @@
         </is>
       </c>
     </row>
-    <row r="180" ht="319" customHeight="1">
+    <row r="180" ht="318.95" customHeight="1">
       <c r="A180" t="inlineStr">
         <is>
           <t>S7-12</t>
@@ -12570,7 +12567,7 @@
         </is>
       </c>
     </row>
-    <row r="181" ht="232" customHeight="1">
+    <row r="181" ht="231.95" customHeight="1">
       <c r="A181" t="inlineStr">
         <is>
           <t>S7-13</t>
@@ -12650,7 +12647,7 @@
         </is>
       </c>
     </row>
-    <row r="183" ht="159.5" customHeight="1">
+    <row r="183" ht="159.6" customHeight="1">
       <c r="A183" t="inlineStr">
         <is>
           <t>S7-15</t>
@@ -12740,7 +12737,7 @@
         </is>
       </c>
     </row>
-    <row r="185" ht="275.5" customHeight="1">
+    <row r="185" ht="275.45" customHeight="1">
       <c r="A185" t="inlineStr">
         <is>
           <t>S7-17</t>
@@ -12785,7 +12782,7 @@
         </is>
       </c>
     </row>
-    <row r="186" ht="203" customHeight="1">
+    <row r="186" ht="203.1" customHeight="1">
       <c r="A186" t="inlineStr">
         <is>
           <t>S7-18</t>
@@ -12861,7 +12858,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>РМНЦ им. Цыба</t>
+          <t>МРНЦ им. А.Ф. Цыба</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -12875,7 +12872,7 @@
         </is>
       </c>
     </row>
-    <row r="188" ht="232" customHeight="1">
+    <row r="188" ht="231.95" customHeight="1">
       <c r="A188" t="inlineStr">
         <is>
           <t>S7-20</t>
@@ -12906,7 +12903,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>РМНЦ им. Цыба</t>
+          <t>МРНЦ им. А.Ф. Цыба</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -12920,7 +12917,7 @@
         </is>
       </c>
     </row>
-    <row r="189" ht="246.5" customHeight="1">
+    <row r="189" ht="246.6" customHeight="1">
       <c r="A189" t="inlineStr">
         <is>
           <t>S7-21</t>
@@ -13010,7 +13007,7 @@
         </is>
       </c>
     </row>
-    <row r="191" ht="159.5" customHeight="1">
+    <row r="191" ht="159.6" customHeight="1">
       <c r="A191" t="inlineStr">
         <is>
           <t>S7-23</t>
@@ -13102,10 +13099,10 @@
     </row>
     <row r="193" ht="261" customHeight="1"/>
     <row r="194" ht="261" customHeight="1"/>
-    <row r="195" ht="290" customHeight="1"/>
-    <row r="196" ht="232" customHeight="1"/>
+    <row r="195" ht="290.1" customHeight="1"/>
+    <row r="196" ht="231.95" customHeight="1"/>
     <row r="197" ht="174" customHeight="1"/>
-    <row r="198" ht="246.5" customHeight="1"/>
+    <row r="198" ht="246.6" customHeight="1"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J2:J499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -13123,7 +13120,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -13197,7 +13194,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="188.5" customHeight="1">
+    <row r="2" ht="188.45" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>POST-01</t>
@@ -13229,7 +13226,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="101.5" customHeight="1">
+    <row r="3" ht="101.45" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>POST-02</t>
@@ -13261,7 +13258,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="101.5" customHeight="1">
+    <row r="4" ht="101.45" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>POST-03</t>
@@ -13399,7 +13396,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="203" customHeight="1">
+    <row r="8" ht="203.1" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>POST-07</t>
@@ -13436,7 +13433,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="159.5" customHeight="1">
+    <row r="9" ht="159.6" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>POST-08</t>
@@ -13473,7 +13470,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="101.5" customHeight="1">
+    <row r="10" ht="101.45" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>POST-09</t>
@@ -13505,7 +13502,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="101.5" customHeight="1">
+    <row r="11" ht="101.45" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>POST-10</t>
@@ -13616,7 +13613,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="232" customHeight="1">
+    <row r="14" ht="231.95" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>POST-13</t>
@@ -13685,7 +13682,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="159.5" customHeight="1">
+    <row r="16" ht="159.6" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>POST-15</t>
@@ -13722,7 +13719,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="116" customHeight="1">
+    <row r="17" ht="116.1" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>POST-16</t>
@@ -13759,7 +13756,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="145" customHeight="1">
+    <row r="18" ht="144.95" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>POST-17</t>
@@ -13796,7 +13793,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="188.5" customHeight="1">
+    <row r="19" ht="188.45" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>POST-18</t>
@@ -13833,7 +13830,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="101.5" customHeight="1">
+    <row r="20" ht="101.45" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>POST-19</t>
@@ -13865,7 +13862,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="145" customHeight="1">
+    <row r="21" ht="144.95" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>POST-20</t>
@@ -13897,7 +13894,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="319" customHeight="1">
+    <row r="22" ht="318.95" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>POST-21</t>
@@ -13934,7 +13931,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="203" customHeight="1">
+    <row r="23" ht="203.1" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>POST-22</t>
@@ -13966,7 +13963,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="290" customHeight="1">
+    <row r="24" ht="290.1" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>POST-23</t>
@@ -13998,7 +13995,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="232" customHeight="1">
+    <row r="25" ht="231.95" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>POST-24</t>
@@ -14030,7 +14027,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="290" customHeight="1">
+    <row r="26" ht="290.1" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>POST-25</t>
@@ -14136,7 +14133,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="246.5" customHeight="1">
+    <row r="29" ht="246.6" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>POST-28</t>
@@ -14210,7 +14207,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="232" customHeight="1">
+    <row r="31" ht="231.95" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>POST-30</t>
@@ -14247,7 +14244,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="203" customHeight="1">
+    <row r="32" ht="203.1" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>POST-31</t>
@@ -14284,7 +14281,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="203" customHeight="1">
+    <row r="33" ht="203.1" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>POST-32</t>
@@ -14321,7 +14318,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="246.5" customHeight="1">
+    <row r="34" ht="246.6" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>POST-33</t>
@@ -14358,7 +14355,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="290" customHeight="1">
+    <row r="35" ht="290.1" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>POST-34</t>
@@ -14390,7 +14387,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="159.5" customHeight="1">
+    <row r="36" ht="159.6" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>POST-35</t>
@@ -14427,7 +14424,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="290" customHeight="1">
+    <row r="37" ht="290.1" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>POST-36</t>
@@ -14464,7 +14461,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="145" customHeight="1">
+    <row r="38" ht="144.95" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>POST-37</t>
@@ -14575,7 +14572,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="145" customHeight="1">
+    <row r="41" ht="144.95" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>POST-40</t>
@@ -14612,7 +14609,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="145" customHeight="1">
+    <row r="42" ht="144.95" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>POST-41</t>
@@ -14649,7 +14646,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="232" customHeight="1">
+    <row r="43" ht="231.95" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
           <t>POST-42</t>
@@ -14686,7 +14683,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="232" customHeight="1">
+    <row r="44" ht="231.95" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
           <t>POST-43</t>
@@ -14787,7 +14784,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="232" customHeight="1">
+    <row r="47" ht="231.95" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
           <t>POST-46</t>
@@ -14819,7 +14816,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="116" customHeight="1">
+    <row r="48" ht="116.1" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
           <t>POST-47</t>
@@ -14868,7 +14865,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="3"/>
@@ -14892,7 +14889,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
+      <c r="A2" s="6" t="n">
         <v>46279.71037037037</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -14937,7 +14934,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="8" t="n">
         <v>46280.72569444445</v>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>

<commit_message>
Update README.md to clarify chair responsibilities for sections and plenary sessions; enhance inconsistency documentation regarding section chairs; modify app.js to support multiple chairs display; increment versioning in index.html and sw.js for cache management consistency.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -78,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -94,6 +95,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1787,6 +1789,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>И. Н. Изосимов</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>I. N. Izosimov</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1818,6 +1830,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>И. А. Митропольский</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>I. A. Mitropolsky</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1827,7 +1849,7 @@
         <v>0.6770833333333334</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.75</v>
+        <v>0.7395833333333334</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1841,12 +1863,22 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1-7</t>
+          <t>1-6</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>117л</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>А. А. Дзюба</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>A. A. Dzyuba</t>
         </is>
       </c>
     </row>
@@ -1880,6 +1912,16 @@
           <t>315л</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>В. О. Сабуров</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>V. O. Saburov</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2295,6 +2337,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>И. А. Мазур</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>I. A. Mazur</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2326,6 +2378,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>А. С. Демьянова</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>A. S. Demyanova</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2357,6 +2419,16 @@
           <t>117л</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Г. А. Феофилов</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>G. A. Feofilov</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2388,6 +2460,16 @@
           <t>315л</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>О. В. Белов</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>O. V. Belov</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2445,6 +2527,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>А. С. Демьянова</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>A. S. Demyanova</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2476,6 +2568,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>В. И. Жеребчевский</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>V. I. Zherebchevsky</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2507,6 +2609,16 @@
           <t>117л</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Д. Прохорова</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>D. Prokhorova</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2538,6 +2650,16 @@
           <t>315л</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>А. П. Черняев</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>A. P. Chernyaev</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2958,6 +3080,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Д. М. Родкин</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>D. M. Rodkin</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2989,6 +3121,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Д. Е. Любашевский</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>D. E. Lyubashevsky</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -3020,6 +3162,16 @@
           <t>117л</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>А. И. Мазур</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>A. I. Mazur</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -3051,6 +3203,16 @@
           <t>315л</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>А. С. Чепурнов</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>A. S. Chepurnov</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3108,16 +3270,8 @@
           <t>холл2</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Время уточняется</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>Time to be confirmed</t>
-        </is>
-      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3927,6 +4081,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>О. А. Рубцова</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>O. A. Rubtsova</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3958,6 +4122,16 @@
           <t>235ц</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>М. А. Науменко</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>M. A. Naumenko</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3989,6 +4163,16 @@
           <t>117л</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>А. В. Канцырев</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>A. V. Kantsyrev</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -4020,6 +4204,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>А. А. Зайцев</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>A. A. Zaitsev</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -4077,6 +4271,16 @@
           <t>117л</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>А. В. Канцырев</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>A. V. Kantsyrev</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -4108,6 +4312,16 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>А. А. Зайцев</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>A. A. Zaitsev</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -4137,6 +4351,16 @@
       <c r="I79" t="inlineStr">
         <is>
           <t>315л</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>С. Мамаева</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>S. Mamaeva</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S192"/>
+  <dimension ref="A1:S191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9227,7 +9451,7 @@
     <row r="105" ht="318.95" customHeight="1">
       <c r="A105" t="inlineStr">
         <is>
-          <t>S3-07</t>
+          <t>S3-08</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -9236,43 +9460,43 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Мальцев</t>
+          <t>Семенов</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Николай</t>
+          <t>Сергей</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Владимирович</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>НИЦ КИ</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>n.maltsev@spbu.ru</t>
+          <t>kindr_cool@mail.ru</t>
         </is>
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>Особенности изучения свойств пучков тяжёлых ионов высоких энергий</t>
+          <t>Критический стенд «П»: современное состояние, особенности и роль исследований для развития технологии ВВЭР</t>
         </is>
       </c>
     </row>
     <row r="106" ht="333.6" customHeight="1">
       <c r="A106" t="inlineStr">
         <is>
-          <t>S3-08</t>
+          <t>S3-09</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9281,43 +9505,38 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Семенов</t>
+          <t>Бурякова</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Сергей</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>Владимирович</t>
+          <t>Елена</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>НИЦ КИ</t>
+          <t>ВНИИЭф</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>kindr_cool@mail.ru</t>
+          <t>suyazova.elena@mail.ru</t>
         </is>
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
-          <t>Критический стенд «П»: современное состояние, особенности и роль исследований для развития технологии ВВЭР</t>
+          <t>Результаты экспериментов с тепловыми трубами с цезиевым теплоносителем</t>
         </is>
       </c>
     </row>
     <row r="107" ht="144.95" customHeight="1">
       <c r="A107" t="inlineStr">
         <is>
-          <t>S3-09</t>
+          <t>S3-10</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9326,38 +9545,43 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Бурякова</t>
+          <t>Розов</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Елена</t>
+          <t>Сергей</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Владимирович</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>ВНИИЭф</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>suyazova.elena@mail.ru</t>
+          <t>rozovs@jinr.ru</t>
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>Результаты экспериментов с тепловыми трубами с цезиевым теплоносителем</t>
+          <t>Низкофоновый детектор нейтронов на основе гелия-3</t>
         </is>
       </c>
     </row>
     <row r="108" ht="246.6" customHeight="1">
       <c r="A108" t="inlineStr">
         <is>
-          <t>S3-10</t>
+          <t>S3-11</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9366,43 +9590,43 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Розов</t>
+          <t>Каретников</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Максим</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Владимирович</t>
+          <t>Донатович</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ВНИИА</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>rozovs@jinr.ru</t>
+          <t>mcsym01@gmail.com</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
-          <t>Низкофоновый детектор нейтронов на основе гелия-3</t>
+          <t>Нейтрон-нейтронные методы дистанционного контроля с использованием меченых нейтронов</t>
         </is>
       </c>
     </row>
     <row r="109" ht="144.95" customHeight="1">
       <c r="A109" t="inlineStr">
         <is>
-          <t>S3-11</t>
+          <t>S3-12</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9411,43 +9635,38 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Каретников</t>
+          <t>Данилкин</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Максим</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>Донатович</t>
+          <t>Владислав</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>ВНИИА</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>mcsym01@gmail.com</t>
+          <t>donyvlad@gmail.com</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>Нейтрон-нейтронные методы дистанционного контроля с использованием меченых нейтронов</t>
+          <t>Моделирование ионной оптики сепаратора STAR с помощью программы SHEMAT</t>
         </is>
       </c>
     </row>
     <row r="110" ht="275.45" customHeight="1">
       <c r="A110" t="inlineStr">
         <is>
-          <t>S3-12</t>
+          <t>S3-13</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9456,16 +9675,21 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Данилкин</t>
+          <t>Веденеев</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Владислав</t>
+          <t>Вячеслав</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Юрьевич</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9475,19 +9699,19 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>donyvlad@gmail.com</t>
+          <t>vvedeneyev@gmail.com</t>
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr">
         <is>
-          <t>Моделирование ионной оптики сепаратора STAR с помощью программы SHEMAT</t>
+          <t>Криогенная газовая ячейка охлаждения ионов. Особенности конструкции, вакуумная система, система газового обеспечения, система охлаждения</t>
         </is>
       </c>
     </row>
     <row r="111" ht="188.45" customHeight="1">
       <c r="A111" t="inlineStr">
         <is>
-          <t>S3-13</t>
+          <t>S3-14</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9496,21 +9720,21 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Веденеев</t>
+          <t>Новоселов</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Вячеслав</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Юрьевич</t>
+          <t>Сергеевич</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9520,19 +9744,19 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>vvedeneyev@gmail.com</t>
+          <t>noval@jinr.ru</t>
         </is>
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>Криогенная газовая ячейка охлаждения ионов. Особенности конструкции, вакуумная система, система газового обеспечения, система охлаждения</t>
+          <t>Измерение времени экстракции ионов из криогенной газовой ячейки охлаждения</t>
         </is>
       </c>
     </row>
     <row r="112" ht="116.1" customHeight="1">
       <c r="A112" t="inlineStr">
         <is>
-          <t>S3-14</t>
+          <t>S3-15</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9541,21 +9765,16 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Новоселов</t>
+          <t>Зимин</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Алексей</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>Сергеевич</t>
+          <t>Илья</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -9565,19 +9784,19 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>noval@jinr.ru</t>
+          <t>zimin@jinr.ru</t>
         </is>
       </c>
       <c r="I112" s="4" t="inlineStr">
         <is>
-          <t>Измерение времени экстракции ионов из криогенной газовой ячейки охлаждения</t>
+          <t>Нейтронные сцинтилляторы на основе кристалла ZnS(Ag)</t>
         </is>
       </c>
     </row>
     <row r="113" ht="246.6" customHeight="1">
       <c r="A113" t="inlineStr">
         <is>
-          <t>S3-15</t>
+          <t>S3-16</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -9586,16 +9805,21 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Зимин</t>
+          <t>Сидорова</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Илья</t>
+          <t>Ольга</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Викторовна</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -9605,19 +9829,19 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>zimin@jinr.ru</t>
+          <t>sidorova@jinr.ru</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>Нейтронные сцинтилляторы на основе кристалла ZnS(Ag)</t>
+          <t>Физическая структура кросс-толка гамма-квантов в сферических многодетекторных сцинтилляционных системах</t>
         </is>
       </c>
     </row>
     <row r="114" ht="188.45" customHeight="1">
       <c r="A114" t="inlineStr">
         <is>
-          <t>S3-16</t>
+          <t>S3-17</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -9626,43 +9850,38 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Сидорова</t>
+          <t>Strizhak</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Ольга</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Викторовна</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ИЯИ</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>sidorova@jinr.ru</t>
+          <t>strizhak@inr.ru</t>
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr">
         <is>
-          <t>Физическая структура кросс-толка гамма-квантов в сферических многодетекторных сцинтилляционных системах</t>
+          <t>Performance and light yield of CsI(pure) scintillation module prototypes at LN2 temperature</t>
         </is>
       </c>
     </row>
     <row r="115" ht="333.6" customHeight="1">
       <c r="A115" t="inlineStr">
         <is>
-          <t>S3-17</t>
+          <t>S3-18</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -9671,38 +9890,38 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Strizhak</t>
+          <t>Суслов</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Иван</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>ИЯИ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>strizhak@inr.ru</t>
+          <t>ivsuslov@jinr.ru</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>Performance and light yield of CsI(pure) scintillation module prototypes at LN2 temperature</t>
+          <t>Пласстмассовые сцинтилляторы с возможностью разделения частиц по форме импульса</t>
         </is>
       </c>
     </row>
     <row r="116" ht="203.1" customHeight="1">
       <c r="A116" t="inlineStr">
         <is>
-          <t>S3-18</t>
+          <t>S3-19</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -9711,16 +9930,21 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Суслов</t>
+          <t>Евсеев</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Иван</t>
+          <t>Сергей</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -9730,19 +9954,19 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>ivsuslov@jinr.ru</t>
+          <t>evseevsa@jinr.ru</t>
         </is>
       </c>
       <c r="I116" s="4" t="inlineStr">
         <is>
-          <t>Пласстмассовые сцинтилляторы с возможностью разделения частиц по форме импульса</t>
+          <t>Исследование радиационной стойкости SiC- и Si-детекторов после облучения альфа-частицами</t>
         </is>
       </c>
     </row>
     <row r="117" ht="130.5" customHeight="1">
       <c r="A117" t="inlineStr">
         <is>
-          <t>S3-19</t>
+          <t>S3-20</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -9751,43 +9975,43 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Евсеев</t>
+          <t>Смирнов</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Игорь</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Борисович</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ПИЯФ</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>evseevsa@jinr.ru</t>
+          <t>smirnov_ib@pnpi.nrcki.ru</t>
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>Исследование радиационной стойкости SiC- и Si-детекторов после облучения альфа-частицами</t>
+          <t>Average Spatial Resolution of Detector Layers of Four-Layer Position-Sensitive Detectors</t>
         </is>
       </c>
     </row>
     <row r="118" ht="275.45" customHeight="1">
       <c r="A118" t="inlineStr">
         <is>
-          <t>S3-20</t>
+          <t>S3-21</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -9796,43 +10020,43 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Смирнов</t>
+          <t>Стрекаловский</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Игорь</t>
+          <t>Олег</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Борисович</t>
+          <t>Викторович</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>ПИЯФ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>smirnov_ib@pnpi.nrcki.ru</t>
+          <t>stroleg1@yandex.ru</t>
         </is>
       </c>
       <c r="I118" s="4" t="inlineStr">
         <is>
-          <t>Average Spatial Resolution of Detector Layers of Four-Layer Position-Sensitive Detectors</t>
+          <t>Применение диджитайзеров CAEN-ХХ42 для регистрации заряженных частиц</t>
         </is>
       </c>
     </row>
     <row r="119" ht="203.1" customHeight="1">
       <c r="A119" t="inlineStr">
         <is>
-          <t>S3-21</t>
+          <t>S3-22</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -9841,43 +10065,38 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Стрекаловский</t>
+          <t>Шимко</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Олег</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Викторович</t>
+          <t>Павел</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>stroleg1@yandex.ru</t>
+          <t>pashashimko0306@gmail.com</t>
         </is>
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>Применение диджитайзеров CAEN-ХХ42 для регистрации заряженных частиц</t>
+          <t>Исследование распределения поглощённой дозы в полимерных материалах при облучении ускоренными электронами</t>
         </is>
       </c>
     </row>
     <row r="120" ht="203.1" customHeight="1">
       <c r="A120" t="inlineStr">
         <is>
-          <t>S3-22</t>
+          <t>S3-23</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -9886,38 +10105,38 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Шимко</t>
+          <t>Цыганкова</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Павел</t>
+          <t>Валерия</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СВКНИИ ДВО</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>pashashimko0306@gmail.com</t>
+          <t>tsigankova.valeriya@mail.ru</t>
         </is>
       </c>
       <c r="I120" s="4" t="inlineStr">
         <is>
-          <t>Исследование распределения поглощённой дозы в полимерных материалах при облучении ускоренными электронами</t>
+          <t>Влияние ²²²Rn на расчёт радиоуглеродного возраста древесных углей</t>
         </is>
       </c>
     </row>
     <row r="121" ht="217.5" customHeight="1">
       <c r="A121" t="inlineStr">
         <is>
-          <t>S3-23</t>
+          <t>S3-24</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -9926,38 +10145,43 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Цыганкова</t>
+          <t>Пухаева</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Валерия</t>
+          <t>Нелли</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Ефимовна</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>СВКНИИ ДВО</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>tsigankova.valeriya@mail.ru</t>
+          <t>pukhaeva@jinr.ru</t>
         </is>
       </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
-          <t>Влияние ²²²Rn на расчёт радиоуглеродного возраста древесных углей</t>
+          <t>Nd/ZnS-модифицированные квантовые точки CdZnSeS как нанокомпоненты сцинтилляционных сред для поиска безнейтринного двойного β-распада ¹⁵⁰Nd</t>
         </is>
       </c>
     </row>
     <row r="122" ht="188.45" customHeight="1">
       <c r="A122" t="inlineStr">
         <is>
-          <t>S3-24</t>
+          <t>S3-25</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -9966,7 +10190,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -9995,14 +10219,14 @@
       </c>
       <c r="I122" s="4" t="inlineStr">
         <is>
-          <t>Nd/ZnS-модифицированные квантовые точки CdZnSeS как нанокомпоненты сцинтилляционных сред для поиска безнейтринного двойного β-распада ¹⁵⁰Nd</t>
+          <t>Results of ARFIM experiment setup for applied research of NOSU</t>
         </is>
       </c>
     </row>
     <row r="123" ht="174" customHeight="1">
       <c r="A123" t="inlineStr">
         <is>
-          <t>S3-25</t>
+          <t>S3-26</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -10011,7 +10235,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -10040,14 +10264,14 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>Results of ARFIM experiment setup for applied research of NOSU</t>
+          <t>Neodymium-modified CdZnSeS/ZnS quantum dots: evolution of optical response and evidence limits for core/shell architecture</t>
         </is>
       </c>
     </row>
     <row r="124" ht="261" customHeight="1">
       <c r="A124" t="inlineStr">
         <is>
-          <t>S3-26</t>
+          <t>S3-27</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -10056,83 +10280,83 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Пухаева</t>
+          <t>Петровская</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Нелли</t>
+          <t>Анна</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Ефимовна</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>ОИЯИ</t>
+          <t>Станиславовна</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>pukhaeva@jinr.ru</t>
+          <t>anita3425@yandex.ru</t>
         </is>
       </c>
       <c r="I124" s="4" t="inlineStr">
         <is>
-          <t>Neodymium-modified CdZnSeS/ZnS quantum dots: evolution of optical response and evidence limits for core/shell architecture</t>
+          <t>Перспективы применения сухой ионно-плазменной технологии дезактивации оборудования ЯЭУ из титановых сплавов</t>
         </is>
       </c>
     </row>
     <row r="125" ht="174" customHeight="1">
       <c r="A125" t="inlineStr">
         <is>
-          <t>S3-27</t>
+          <t>S4-01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Петровская</t>
+          <t>Бикметов</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Анна</t>
+          <t>Никита</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Станиславовна</t>
+          <t>Рафальевич</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>anita3425@yandex.ru</t>
+          <t>bikmetov@jinr.ru</t>
         </is>
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>Перспективы применения сухой ионно-плазменной технологии дезактивации оборудования ЯЭУ из титановых сплавов</t>
+          <t>Investigation of nuclear deformation influence on anisotropic flows in heavy-ion collisions at NICA energies</t>
         </is>
       </c>
     </row>
     <row r="126" ht="362.45" customHeight="1">
       <c r="A126" t="inlineStr">
         <is>
-          <t>S4-01</t>
+          <t>S4-02</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -10141,43 +10365,43 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Бикметов</t>
+          <t>Вечернин</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Никита</t>
+          <t>Владимир</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Рафальевич</t>
+          <t>Викторович</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>bikmetov@jinr.ru</t>
+          <t>v.vechernin@spbu.ru</t>
         </is>
       </c>
       <c r="I126" s="4" t="inlineStr">
         <is>
-          <t>Investigation of nuclear deformation influence on anisotropic flows in heavy-ion collisions at NICA energies</t>
+          <t>Кумулятивные явления в области больших поперечных импульсов и их наблюдение в столкновениях ядер на коллайдере NICA</t>
         </is>
       </c>
     </row>
     <row r="127" ht="144.95" customHeight="1">
       <c r="A127" t="inlineStr">
         <is>
-          <t>S4-02</t>
+          <t>S4-03</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -10186,43 +10410,38 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Вечернин</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Владимир</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>Викторович</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>v.vechernin@spbu.ru</t>
+          <t>s.sharma.hep@gmail.com</t>
         </is>
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>Кумулятивные явления в области больших поперечных импульсов и их наблюдение в столкновениях ядер на коллайдере NICA</t>
+          <t>Inclusive J/ψ Production as a Probe of Gluon Dynamics at NICA</t>
         </is>
       </c>
     </row>
     <row r="128" ht="290.1" customHeight="1">
       <c r="A128" t="inlineStr">
         <is>
-          <t>S4-03</t>
+          <t>S4-04</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -10231,38 +10450,43 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Жаров</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Михаил</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Андреевич</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>s.sharma.hep@gmail.com</t>
+          <t>m.zharov@spbu.ru</t>
         </is>
       </c>
       <c r="I128" s="4" t="inlineStr">
         <is>
-          <t>Inclusive J/ψ Production as a Probe of Gluon Dynamics at NICA</t>
+          <t>Моделирование кумулятивных эффектов в столкновениях тяжелых ионов при энергиях коллайдера NICA</t>
         </is>
       </c>
     </row>
     <row r="129" ht="261" customHeight="1">
       <c r="A129" t="inlineStr">
         <is>
-          <t>S4-04</t>
+          <t>S4-05</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -10271,43 +10495,43 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Жаров</t>
+          <t>Идрисов</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Михаил</t>
+          <t>Дим</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Андреевич</t>
+          <t>Маратович</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>m.zharov@spbu.ru</t>
+          <t>idrisov.dim@mail.ru</t>
         </is>
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>Моделирование кумулятивных эффектов в столкновениях тяжелых ионов при энергиях коллайдера NICA</t>
+          <t>Методы определения центральности с использованием передних детекторов в эксперименте BM@N</t>
         </is>
       </c>
     </row>
     <row r="130" ht="231.95" customHeight="1">
       <c r="A130" t="inlineStr">
         <is>
-          <t>S4-05</t>
+          <t>S4-06</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -10316,43 +10540,43 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Идрисов</t>
+          <t>Plotnikov</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Дим</t>
+          <t>Vasilii</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Маратович</t>
+          <t>Alexandrovich</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>idrisov.dim@mail.ru</t>
+          <t>vplotnikov@jinr.ru</t>
         </is>
       </c>
       <c r="I130" s="4" t="inlineStr">
         <is>
-          <t>Методы определения центральности с использованием передних детекторов в эксперименте BM@N</t>
+          <t>Λd сorrelation function in Xe+CsI collisions at 3.8 AGeV in the BM@N experiment</t>
         </is>
       </c>
     </row>
     <row r="131" ht="275.45" customHeight="1">
       <c r="A131" t="inlineStr">
         <is>
-          <t>S4-06</t>
+          <t>S4-07</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -10361,43 +10585,43 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Plotnikov</t>
+          <t>Зубанков</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Vasilii</t>
+          <t>Александр</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Alexandrovich</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>vplotnikov@jinr.ru</t>
+          <t>zubankov@inr.ru</t>
         </is>
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>Λd сorrelation function in Xe+CsI collisions at 3.8 AGeV in the BM@N experiment</t>
+          <t>Measurement of double differential inclusive cross sections of forward neutron emission in the BM@N experiment</t>
         </is>
       </c>
     </row>
     <row r="132" ht="130.5" customHeight="1">
       <c r="A132" t="inlineStr">
         <is>
-          <t>S4-07</t>
+          <t>S4-08</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -10406,43 +10630,43 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Зубанков</t>
+          <t>Андронов</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Александр</t>
+          <t>Евгений</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Владимирович</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>zubankov@inr.ru</t>
+          <t>e.v.andronov@spbu.ru</t>
         </is>
       </c>
       <c r="I132" s="4" t="inlineStr">
         <is>
-          <t>Measurement of double differential inclusive cross sections of forward neutron emission in the BM@N experiment</t>
+          <t>Influence of colour string configurations on rapidity multiplicity correlations</t>
         </is>
       </c>
     </row>
     <row r="133" ht="246.6" customHeight="1">
       <c r="A133" t="inlineStr">
         <is>
-          <t>S4-08</t>
+          <t>S4-10</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -10450,17 +10674,19 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C133" t="n">
-        <v>8</v>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Андронов</t>
+          <t>Герасименюк</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Евгений</t>
+          <t>Николай</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -10470,24 +10696,24 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>e.v.andronov@spbu.ru</t>
+          <t>gerasimenyuk.nv@dvfu.ru</t>
         </is>
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>Influence of colour string configurations on rapidity multiplicity correlations</t>
+          <t>Экранирование заряда в многокомпонентной аблелевой модели Хиггса</t>
         </is>
       </c>
     </row>
     <row r="134" ht="217.5" customHeight="1">
       <c r="A134" t="inlineStr">
         <is>
-          <t>S4-10</t>
+          <t>S4-11</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -10497,44 +10723,44 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Герасименюк</t>
+          <t>Зайцев</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Николай</t>
+          <t>Андрей</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Владимирович</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>ДВФУ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>gerasimenyuk.nv@dvfu.ru</t>
+          <t>zaicev@jinr.ru</t>
         </is>
       </c>
       <c r="I134" s="4" t="inlineStr">
         <is>
-          <t>Экранирование заряда в многокомпонентной аблелевой модели Хиггса</t>
+          <t>Ядро ⁸Be и состояние Хойла в диссоциации релятивистских ядер</t>
         </is>
       </c>
     </row>
     <row r="135" ht="188.45" customHeight="1">
       <c r="A135" t="inlineStr">
         <is>
-          <t>S4-11</t>
+          <t>S4-12</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -10544,44 +10770,44 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Зайцев</t>
+          <t>Скородько</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Андрей</t>
+          <t>Татьяна</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Юрьевна</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>zaicev@jinr.ru</t>
+          <t>tatiskor@mail.ru</t>
         </is>
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>Ядро ⁸Be и состояние Хойла в диссоциации релятивистских ядер</t>
+          <t>Dibaryon d*(2380) : prediction, detection, understanding</t>
         </is>
       </c>
     </row>
     <row r="136" ht="246.6" customHeight="1">
       <c r="A136" t="inlineStr">
         <is>
-          <t>S4-12</t>
+          <t>S4-14</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -10591,44 +10817,44 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Скородько</t>
+          <t>Friesen</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Татьяна</t>
+          <t>Alexandra</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Юрьевна</t>
+          <t>Vadimovna</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>tatiskor@mail.ru</t>
+          <t>avfriesen@theor.jinr.ru</t>
         </is>
       </c>
       <c r="I136" s="4" t="inlineStr">
         <is>
-          <t>Dibaryon d*(2380) : prediction, detection, understanding</t>
+          <t>Mass spectrum of noncharmed and charmed meson states at finite temperature in extended linear-sigma model</t>
         </is>
       </c>
     </row>
     <row r="137" ht="174" customHeight="1">
       <c r="A137" t="inlineStr">
         <is>
-          <t>S4-14</t>
+          <t>S4-15</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -10636,24 +10862,22 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="C137" t="n">
+        <v>15</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Friesen</t>
+          <t>Авдеев</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Alexandra</t>
+          <t>Сергей</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Vadimovna</t>
+          <t>Петрович</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -10663,19 +10887,19 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>avfriesen@theor.jinr.ru</t>
+          <t>avdeyev@jinr.ru</t>
         </is>
       </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
-          <t>Mass spectrum of noncharmed and charmed meson states at finite temperature in extended linear-sigma model</t>
+          <t>Source velocity in collisions of 2.1 GeV and 3.6 GeV protons with gold target.</t>
         </is>
       </c>
     </row>
     <row r="138" ht="246.6" customHeight="1">
       <c r="A138" t="inlineStr">
         <is>
-          <t>S4-15</t>
+          <t>S4-16</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -10684,43 +10908,43 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Авдеев</t>
+          <t>Иванищев</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Дмитрий</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Петрович</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>НИЦ КИ-ПИЯФ</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>avdeyev@jinr.ru</t>
+          <t>ivanishchev_da@pnpi.nrcki.ru</t>
         </is>
       </c>
       <c r="I138" s="4" t="inlineStr">
         <is>
-          <t>Source velocity in collisions of 2.1 GeV and 3.6 GeV protons with gold target.</t>
+          <t>Особенности измерения свойств резонансов в эксперименте MPD в Xe+W столкновениях при энергии 2,5 A*ГэВ</t>
         </is>
       </c>
     </row>
     <row r="139" ht="174" customHeight="1">
       <c r="A139" t="inlineStr">
         <is>
-          <t>S4-16</t>
+          <t>S4-17</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -10729,43 +10953,43 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Иванищев</t>
+          <t>Силагадзе</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Дмитрий</t>
+          <t>Зураб</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Карлоевич</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>НИЦ КИ-ПИЯФ</t>
+          <t>ИЯФ Новосиб</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>ivanishchev_da@pnpi.nrcki.ru</t>
+          <t>silagadze@inp.nsk.su</t>
         </is>
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>Особенности измерения свойств резонансов в эксперименте MPD в Xe+W столкновениях при энергии 2,5 A*ГэВ</t>
+          <t>Pauli equation in spaces of constant curvature and extended Nikiforov-Uvarov method</t>
         </is>
       </c>
     </row>
     <row r="140" ht="144.95" customHeight="1">
       <c r="A140" t="inlineStr">
         <is>
-          <t>S4-17</t>
+          <t>S4-18</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -10774,43 +10998,43 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Силагадзе</t>
+          <t>Феофилов</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Зураб</t>
+          <t>Григорий</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Карлоевич</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>ИЯФ Новосиб</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>silagadze@inp.nsk.su</t>
+          <t>g.feofilov@spbu.ru</t>
         </is>
       </c>
       <c r="I140" s="4" t="inlineStr">
         <is>
-          <t>Pauli equation in spaces of constant curvature and extended Nikiforov-Uvarov method</t>
+          <t>Минимизация объемных флуктуаций при поиске критической точки сильно взаимодействующей материи в релятивистских ядерных столкновениях</t>
         </is>
       </c>
     </row>
     <row r="141" ht="144.95" customHeight="1">
       <c r="A141" t="inlineStr">
         <is>
-          <t>S4-18</t>
+          <t>S4-19</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -10819,43 +11043,38 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Феофилов</t>
+          <t>Prokhorova</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Григорий</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>Александрович</t>
+          <t>Daria</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>Tsinghua Univ., China</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>g.feofilov@spbu.ru</t>
+          <t>daria-prokhorova@mail.tsinghua.edu.cn</t>
         </is>
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>Минимизация объемных флуктуаций при поиске критической точки сильно взаимодействующей материи в релятивистских ядерных столкновениях</t>
+          <t>Heavy-flavor jet quenching in pre-equilibrium medium</t>
         </is>
       </c>
     </row>
     <row r="142" ht="174" customHeight="1">
       <c r="A142" t="inlineStr">
         <is>
-          <t>S4-19</t>
+          <t>S4-20</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -10864,38 +11083,43 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Prokhorova</t>
+          <t>Недорезов</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Daria</t>
+          <t>Егор</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Вячеславович</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Tsinghua Univ., China</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>daria-prokhorova@mail.tsinghua.edu.cn</t>
+          <t>nedorezov@jinr.ru</t>
         </is>
       </c>
       <c r="I142" s="4" t="inlineStr">
         <is>
-          <t>Heavy-flavor jet quenching in pre-equilibrium medium</t>
+          <t>Overview of the STAR hot QCD results</t>
         </is>
       </c>
     </row>
     <row r="143" ht="231.95" customHeight="1">
       <c r="A143" t="inlineStr">
         <is>
-          <t>S4-20</t>
+          <t>S4-21</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -10904,43 +11128,43 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Недорезов</t>
+          <t>Ануфриев</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Егор</t>
+          <t>Антон</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Вячеславович</t>
+          <t>Витальевич</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>nedorezov@jinr.ru</t>
+          <t>antonman200@yandex.ru</t>
         </is>
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>Overview of the STAR hot QCD results</t>
+          <t>Исследование выходов заряженных адронов в рамках гидродинамического моделирования с применением голографического уравнения состояния</t>
         </is>
       </c>
     </row>
     <row r="144" ht="159.6" customHeight="1">
       <c r="A144" t="inlineStr">
         <is>
-          <t>S4-21</t>
+          <t>S4-22</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -10949,21 +11173,21 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Ануфриев</t>
+          <t>Галактионов</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Антон</t>
+          <t>Кирилл</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Витальевич</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -10973,19 +11197,19 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>antonman200@yandex.ru</t>
+          <t>kirill.galaktionov@spbu.ru</t>
         </is>
       </c>
       <c r="I144" s="4" t="inlineStr">
         <is>
-          <t>Исследование выходов заряженных адронов в рамках гидродинамического моделирования с применением голографического уравнения состояния</t>
+          <t>Исследование нейросетевых подходов к оценке прицельного параметра в столкновениях тяжелых ионов на основе 4π информации о событии</t>
         </is>
       </c>
     </row>
     <row r="145" ht="246.6" customHeight="1">
       <c r="A145" t="inlineStr">
         <is>
-          <t>S4-22</t>
+          <t>S4-23</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -10994,43 +11218,43 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Галактионов</t>
+          <t>Дьяченко</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Кирилл</t>
+          <t>Александр</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Трофимович</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>НИЦ КИ-ПИЯФ</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>kirill.galaktionov@spbu.ru</t>
+          <t>dyachenko_a@mail.ru</t>
         </is>
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>Исследование нейросетевых подходов к оценке прицельного параметра в столкновениях тяжелых ионов на основе 4π информации о событии</t>
+          <t>Неравновесный квантовый гидродинамический подход и эмиссия фрагментов в столкновениях тяжелых ионов промежуточных энергий</t>
         </is>
       </c>
     </row>
     <row r="146" ht="203.1" customHeight="1">
       <c r="A146" t="inlineStr">
         <is>
-          <t>S4-23</t>
+          <t>S4-24</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -11039,43 +11263,43 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Дьяченко</t>
+          <t>Белокурова</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Александр</t>
+          <t>Светлана</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Трофимович</t>
+          <t>Николаевна</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>НИЦ КИ-ПИЯФ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>dyachenko_a@mail.ru</t>
+          <t>s.belokurova@spbu.ru</t>
         </is>
       </c>
       <c r="I146" s="4" t="inlineStr">
         <is>
-          <t>Неравновесный квантовый гидродинамический подход и эмиссия фрагментов в столкновениях тяжелых ионов промежуточных энергий</t>
+          <t>Применение классического глауберовского подхода к описанию дейтрон-дейтронного взаимодействия</t>
         </is>
       </c>
     </row>
     <row r="147" ht="318.95" customHeight="1">
       <c r="A147" t="inlineStr">
         <is>
-          <t>S4-24</t>
+          <t>S4-25</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -11084,21 +11308,21 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Белокурова</t>
+          <t>Размыслов</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Светлана</t>
+          <t>Константин</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Николаевна</t>
+          <t>Владимирович</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -11108,19 +11332,19 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>s.belokurova@spbu.ru</t>
+          <t>yoitz@yandex.ru</t>
         </is>
       </c>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>Применение классического глауберовского подхода к описанию дейтрон-дейтронного взаимодействия</t>
+          <t>О применении генераторов EPOS4, UrQMD, PHQMD и PYTHIA для анализа событий в физике сверхвысоких энергий</t>
         </is>
       </c>
     </row>
     <row r="148" ht="130.5" customHeight="1">
       <c r="A148" t="inlineStr">
         <is>
-          <t>S4-25</t>
+          <t>S4-26</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -11129,43 +11353,43 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Размыслов</t>
+          <t>Мягков</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Константин</t>
+          <t>Данила</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Владимирович</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>НИИЯФ МГУ</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>yoitz@yandex.ru</t>
+          <t>danila.myagkov.msu@mail.ru</t>
         </is>
       </c>
       <c r="I148" s="4" t="inlineStr">
         <is>
-          <t>О применении генераторов EPOS4, UrQMD, PHQMD и PYTHIA для анализа событий в физике сверхвысоких энергий</t>
+          <t>Моделирование влияния деформации ядер на азимутальную анизотропию частиц в генераторе событий HYDJET++</t>
         </is>
       </c>
     </row>
     <row r="149" ht="72.59999999999999" customHeight="1">
       <c r="A149" t="inlineStr">
         <is>
-          <t>S4-26</t>
+          <t>S4-27</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -11174,43 +11398,38 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Мягков</t>
+          <t>Vasilieva</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Данила</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>Александрович</t>
+          <t>Anastasiia</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>НИИЯФ МГУ</t>
+          <t>МИФИ</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>danila.myagkov.msu@mail.ru</t>
+          <t>anastasiyavasileva00@gmail.com</t>
         </is>
       </c>
       <c r="I149" s="4" t="inlineStr">
         <is>
-          <t>Моделирование влияния деформации ядер на азимутальную анизотропию частиц в генераторе событий HYDJET++</t>
+          <t>Analysis of charged and identified hadron spectra with Tsallis distributions in O+O, Kr+Kr, and Xe+Xe collisions at √sₙₙ = 6 GeV using the UrQMD model</t>
         </is>
       </c>
     </row>
     <row r="150" ht="348" customHeight="1">
       <c r="A150" t="inlineStr">
         <is>
-          <t>S4-27</t>
+          <t>S4-28</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -11219,83 +11438,88 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Vasilieva</t>
+          <t>Калугин</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Anastasiia</t>
+          <t>Никита</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Константинович</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>МИФИ</t>
+          <t>КИ ИФВЭ</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>anastasiyavasileva00@gmail.com</t>
+          <t>Nikita.Kalugin@ihep.ru</t>
         </is>
       </c>
       <c r="I150" s="4" t="inlineStr">
         <is>
-          <t>Analysis of charged and identified hadron spectra with Tsallis distributions in O+O, Kr+Kr, and Xe+Xe collisions at √sₙₙ = 6 GeV using the UrQMD model</t>
+          <t>Измерение выстроенности K*⁻(892)-мезонов, образованных в каон-ядерных и пион-ядерных взаимодействиях на ускорительном комплексе У-70</t>
         </is>
       </c>
     </row>
     <row r="151" ht="318.95" customHeight="1">
       <c r="A151" t="inlineStr">
         <is>
-          <t>S4-28</t>
+          <t>S5-01</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Калугин</t>
+          <t>Чернышев</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Никита</t>
+          <t>Борис</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Константинович</t>
+          <t>Андреевич</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>КИ ИФВЭ</t>
+          <t>МИФИ</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Nikita.Kalugin@ihep.ru</t>
+          <t>chernyshev@mephi.ru</t>
         </is>
       </c>
       <c r="I151" s="4" t="inlineStr">
         <is>
-          <t>Измерение выстроенности K*⁻(892)-мезонов, образованных в каон-ядерных и пион-ядерных взаимодействиях на ускорительном комплексе У-70</t>
+          <t>Поиск тринейтрона в реакциях поглощения остановившихся пионов ядрами ⁹Be</t>
         </is>
       </c>
     </row>
     <row r="152" ht="290.1" customHeight="1">
       <c r="A152" t="inlineStr">
         <is>
-          <t>S5-01</t>
+          <t>S5-02</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -11304,43 +11528,43 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Чернышев</t>
+          <t>Борзаков</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Борис</t>
+          <t>Сергей</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Андреевич</t>
+          <t>Борисович</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>МИФИ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>chernyshev@mephi.ru</t>
+          <t>sbor@nf.jinr.ru</t>
         </is>
       </c>
       <c r="I152" s="4" t="inlineStr">
         <is>
-          <t>Поиск тринейтрона в реакциях поглощения остановившихся пионов ядрами ⁹Be</t>
+          <t>Возможное существование синглетного дейтрона как дибарионного резонанса и проблема существования динейтрона</t>
         </is>
       </c>
     </row>
     <row r="153" ht="246.6" customHeight="1">
       <c r="A153" t="inlineStr">
         <is>
-          <t>S5-02</t>
+          <t>S5-03</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -11349,43 +11573,43 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Борзаков</t>
+          <t>Ефименко</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Мария</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Борисович</t>
+          <t>Константиновна</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>ТОГУ</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>sbor@nf.jinr.ru</t>
+          <t>ef.maria97@yandex.ru</t>
         </is>
       </c>
       <c r="I153" s="4" t="inlineStr">
         <is>
-          <t>Возможное существование синглетного дейтрона как дибарионного резонанса и проблема существования динейтрона</t>
+          <t>Excited states of ⁶He nucleus in the SS-HORSE–NCSM approach</t>
         </is>
       </c>
     </row>
     <row r="154" ht="261" customHeight="1">
       <c r="A154" t="inlineStr">
         <is>
-          <t>S5-03</t>
+          <t>S5-04</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -11394,21 +11618,21 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Ефименко</t>
+          <t>Зайцев</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Мария</t>
+          <t>Сергей</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Константиновна</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -11418,19 +11642,19 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>ef.maria97@yandex.ru</t>
+          <t>000282@togudv.ru</t>
         </is>
       </c>
       <c r="I154" s="4" t="inlineStr">
         <is>
-          <t>Excited states of ⁶He nucleus in the SS-HORSE–NCSM approach</t>
+          <t>Ионизация атомов протонным ударом в представлении параболических квазиштурмовских функций</t>
         </is>
       </c>
     </row>
     <row r="155" ht="261" customHeight="1">
       <c r="A155" t="inlineStr">
         <is>
-          <t>S5-04</t>
+          <t>S5-05</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -11439,7 +11663,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -11448,12 +11672,12 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Александр</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Сергеевич</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -11463,19 +11687,19 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>000282@togudv.ru</t>
+          <t>alzaytsev@togudv.ru</t>
         </is>
       </c>
       <c r="I155" s="4" t="inlineStr">
         <is>
-          <t>Ионизация атомов протонным ударом в представлении параболических квазиштурмовских функций</t>
+          <t>Атом водорода в поле лазерного импульса в представлении параболических волновых пакетов</t>
         </is>
       </c>
     </row>
     <row r="156" ht="348" customHeight="1">
       <c r="A156" t="inlineStr">
         <is>
-          <t>S5-05</t>
+          <t>S5-06</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -11484,43 +11708,38 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Зайцев</t>
+          <t>Шалапинин</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Александр</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>Сергеевич</t>
+          <t>Денис</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>ТОГУ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>alzaytsev@togudv.ru</t>
+          <t>shalapinin@theor.jinr.ru</t>
         </is>
       </c>
       <c r="I156" s="4" t="inlineStr">
         <is>
-          <t>Атом водорода в поле лазерного импульса в представлении параболических волновых пакетов</t>
+          <t>Van der Waals dimers of neon</t>
         </is>
       </c>
     </row>
     <row r="157" ht="304.5" customHeight="1">
       <c r="A157" t="inlineStr">
         <is>
-          <t>S5-06</t>
+          <t>S5-07</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -11529,38 +11748,43 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Шалапинин</t>
+          <t>Рубцова</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Денис</t>
+          <t>Ольга</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Андреевна</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>НИИЯФ</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>shalapinin@theor.jinr.ru</t>
+          <t>rubtsova-olga@yandex.ru</t>
         </is>
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>Van der Waals dimers of neon</t>
+          <t>Finding virtual states via wave-packet continuum discretization</t>
         </is>
       </c>
     </row>
     <row r="158" ht="188.45" customHeight="1">
       <c r="A158" t="inlineStr">
         <is>
-          <t>S5-07</t>
+          <t>S5-08</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -11569,43 +11793,43 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Рубцова</t>
+          <t>Мотовилов</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Ольга</t>
+          <t>Александр</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Андреевна</t>
+          <t>Константинович</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>НИИЯФ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>rubtsova-olga@yandex.ru</t>
+          <t>motovilv@gmail.com</t>
         </is>
       </c>
       <c r="I158" s="4" t="inlineStr">
         <is>
-          <t>Finding virtual states via wave-packet continuum discretization</t>
+          <t>Resonances of a two-particle system on a 1D lattice</t>
         </is>
       </c>
     </row>
     <row r="159" ht="261" customHeight="1">
       <c r="A159" t="inlineStr">
         <is>
-          <t>S5-08</t>
+          <t>S5-09</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -11614,88 +11838,88 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Мотовилов</t>
+          <t>Яковлев</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Александр</t>
+          <t>Сергей</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Константинович</t>
+          <t>Леонидович</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>motovilv@gmail.com</t>
+          <t>s.yakovlev@spbu.ru</t>
         </is>
       </c>
       <c r="I159" s="4" t="inlineStr">
         <is>
-          <t>Resonances of a two-particle system on a 1D lattice</t>
+          <t>3-3 рассеяние в системах трёх частиц с короткодействующими и кулоновскими взаимодействиями</t>
         </is>
       </c>
     </row>
     <row r="160" ht="130.5" customHeight="1">
       <c r="A160" t="inlineStr">
         <is>
-          <t>S5-09</t>
+          <t>S6-01</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Яковлев</t>
+          <t>Дербин</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Сергей</t>
+          <t>Александр</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Леонидович</t>
+          <t>Владимирович</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>ПИЯФ</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>s.yakovlev@spbu.ru</t>
+          <t>derbin_av@pnpi.nrcki.ru</t>
         </is>
       </c>
       <c r="I160" s="4" t="inlineStr">
         <is>
-          <t>3-3 рассеяние в системах трёх частиц с короткодействующими и кулоновскими взаимодействиями</t>
+          <t>Поиск тяжелого стерильного нейтрино в бета-распаде ¹⁴⁴Pr</t>
         </is>
       </c>
     </row>
     <row r="161" ht="246.6" customHeight="1">
       <c r="A161" t="inlineStr">
         <is>
-          <t>S6-01</t>
+          <t>S6-02</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -11704,43 +11928,43 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Дербин</t>
+          <t>Кондратьев</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Александр</t>
+          <t>Владимир</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Владимирович</t>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>ПИЯФ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>derbin_av@pnpi.nrcki.ru</t>
+          <t>vkondrat@theor.jinr.ru</t>
         </is>
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>Поиск тяжелого стерильного нейтрино в бета-распаде ¹⁴⁴Pr</t>
+          <t>Эффекты динамо и осцилляций в спектрах нейтрино сверхновых</t>
         </is>
       </c>
     </row>
     <row r="162" ht="231.95" customHeight="1">
       <c r="A162" t="inlineStr">
         <is>
-          <t>S6-02</t>
+          <t>S6-03</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -11749,7 +11973,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -11778,14 +12002,14 @@
       </c>
       <c r="I162" s="4" t="inlineStr">
         <is>
-          <t>Эффекты динамо и осцилляций в спектрах нейтрино сверхновых</t>
+          <t>Эффекты намагниченности ядер во взрывном нуклеосинтезе</t>
         </is>
       </c>
     </row>
     <row r="163" ht="57.95" customHeight="1">
       <c r="A163" t="inlineStr">
         <is>
-          <t>S6-03</t>
+          <t>S6-04</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -11794,21 +12018,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Кондратьев</t>
+          <t>Лубашевский</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Владимир</t>
-        </is>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>Николаевич</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -11818,19 +12037,19 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>vkondrat@theor.jinr.ru</t>
+          <t>lubashev@jinr.ru</t>
         </is>
       </c>
       <c r="I163" s="4" t="inlineStr">
         <is>
-          <t>Эффекты намагниченности ядер во взрывном нуклеосинтезе</t>
+          <t>Search for rare processes within the νGeN experiment at Kalinin nuclear power plant</t>
         </is>
       </c>
     </row>
     <row r="164" ht="130.5" customHeight="1">
       <c r="A164" t="inlineStr">
         <is>
-          <t>S6-04</t>
+          <t>S6-05</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -11839,38 +12058,43 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Лубашевский</t>
+          <t>Громов</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Максим</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Борисович</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>НИИЯФ</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>lubashev@jinr.ru</t>
+          <t>gromov@physics.msu.ru</t>
         </is>
       </c>
       <c r="I164" s="4" t="inlineStr">
         <is>
-          <t>Search for rare processes within the νGeN experiment at Kalinin nuclear power plant</t>
+          <t>Precise reactor antineutrino spectrum measurement with TAO detector</t>
         </is>
       </c>
     </row>
     <row r="165" ht="101.45" customHeight="1">
       <c r="A165" t="inlineStr">
         <is>
-          <t>S6-05</t>
+          <t>S6-06</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -11879,21 +12103,21 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Громов</t>
+          <t>Михеев</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Максим</t>
+          <t>Семён</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Борисович</t>
+          <t>Алексеевич</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -11903,19 +12127,19 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>gromov@physics.msu.ru</t>
+          <t>semenmihey@gmail.com</t>
         </is>
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>Precise reactor antineutrino spectrum measurement with TAO detector</t>
+          <t>Условия появления Λ-гиперонов в материи нейтронных звёзд в моделях среднего поля</t>
         </is>
       </c>
     </row>
     <row r="166" ht="217.5" customHeight="1">
       <c r="A166" t="inlineStr">
         <is>
-          <t>S6-06</t>
+          <t>S6-07</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -11924,43 +12148,38 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Михеев</t>
+          <t>Kabir</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Семён</t>
-        </is>
-      </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>Алексеевич</t>
+          <t>Abdul</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>НИИЯФ</t>
+          <t>Institute of Space Technology (Islamabad, Pakistan)</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>semenmihey@gmail.com</t>
+          <t>kabirkhanak1@gmail.com</t>
         </is>
       </c>
       <c r="I166" s="4" t="inlineStr">
         <is>
-          <t>Условия появления Λ-гиперонов в материи нейтронных звёзд в моделях среднего поля</t>
+          <t>Analysis of radiative capture of proton ¹¹B (p, γ) ¹²C at low energy</t>
         </is>
       </c>
     </row>
     <row r="167" ht="144.95" customHeight="1">
       <c r="A167" t="inlineStr">
         <is>
-          <t>S6-07</t>
+          <t>S6-08</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -11969,78 +12188,78 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Kabir</t>
+          <t>Le</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Abdul</t>
+          <t>Huy Viet</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Institute of Space Technology (Islamabad, Pakistan)</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>kabirkhanak1@gmail.com</t>
+          <t>leviethuy1@duytan.edu.vn</t>
         </is>
       </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>Analysis of radiative capture of proton ¹¹B (p, γ) ¹²C at low energy</t>
+          <t>Characterization of the cosmic muon background in the νGeN experiment</t>
         </is>
       </c>
     </row>
     <row r="168" ht="174" customHeight="1">
       <c r="A168" t="inlineStr">
         <is>
-          <t>S6-08</t>
+          <t>S7-01</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Le</t>
+          <t>Киселев</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Huy Viet</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>ОИЯИ</t>
+          <t>Василий</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Алексеевич</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>leviethuy1@duytan.edu.vn</t>
+          <t>kiselevva@fnkcrio.ru</t>
         </is>
       </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>Characterization of the cosmic muon background in the νGeN experiment</t>
+          <t>Подход к оптимизации распределения поглощенной дозы в биологическом объекте в лучевой терапии пучком ускоренных протонов</t>
         </is>
       </c>
     </row>
     <row r="169" ht="144.95" customHeight="1">
       <c r="A169" t="inlineStr">
         <is>
-          <t>S7-01</t>
+          <t>S7-02</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -12049,38 +12268,43 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Киселев</t>
+          <t>Щербаков</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Василий</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Алексеевич</t>
+          <t>Александрович</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>kiselevva@fnkcrio.ru</t>
+          <t>sherbakov.aa15@physics.msu.ru</t>
         </is>
       </c>
       <c r="I169" s="4" t="inlineStr">
         <is>
-          <t>Подход к оптимизации распределения поглощенной дозы в биологическом объекте в лучевой терапии пучком ускоренных протонов</t>
+          <t>Оценка рисков развития радиационно-индуцированных заболеваний при проведении лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="170" ht="188.45" customHeight="1">
       <c r="A170" t="inlineStr">
         <is>
-          <t>S7-02</t>
+          <t>S7-03</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -12089,43 +12313,43 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Щербаков</t>
+          <t>Васильева</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Алина</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Геннадиевна</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>НИЦ КИ ИФВЭ</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>sherbakov.aa15@physics.msu.ru</t>
+          <t>vasilyeva-ag@ihep.ru</t>
         </is>
       </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t>Оценка рисков развития радиационно-индуцированных заболеваний при проведении лучевой терапии</t>
+          <t>Измерение сечения реакции ¹²C(¹²C,X)¹¹C: особенности эксперимента и оценка неопределенностей</t>
         </is>
       </c>
     </row>
     <row r="171" ht="159.6" customHeight="1">
       <c r="A171" t="inlineStr">
         <is>
-          <t>S7-03</t>
+          <t>S7-04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -12134,21 +12358,21 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Васильева</t>
+          <t>Парменова</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Алина</t>
+          <t>Екатерина</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Геннадиевна</t>
+          <t>Владимировна</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -12158,19 +12382,19 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>vasilyeva-ag@ihep.ru</t>
+          <t>Ekaterina.Parmenova@ihep.ru</t>
         </is>
       </c>
       <c r="I171" s="4" t="inlineStr">
         <is>
-          <t>Измерение сечения реакции ¹²C(¹²C,X)¹¹C: особенности эксперимента и оценка неопределенностей</t>
+          <t>Реализация работы с данными КТ в системе планирования ионной лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="172" ht="203.1" customHeight="1">
       <c r="A172" t="inlineStr">
         <is>
-          <t>S7-04</t>
+          <t>S7-05</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -12179,43 +12403,43 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Парменова</t>
+          <t>Петров</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Екатерина</t>
+          <t>Виталий</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Владимировна</t>
+          <t>Валерьевич</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>НИЦ КИ ИФВЭ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Ekaterina.Parmenova@ihep.ru</t>
+          <t>vitalii17@bk.ru</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>Реализация работы с данными КТ в системе планирования ионной лучевой терапии</t>
+          <t>Трекинг, измерение энергии и получение диагностических изображений с использованием кремниевых пиксельных сенсоров</t>
         </is>
       </c>
     </row>
     <row r="173" ht="159.6" customHeight="1">
       <c r="A173" t="inlineStr">
         <is>
-          <t>S7-05</t>
+          <t>S7-06</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -12224,43 +12448,43 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Петров</t>
+          <t>Мерзликин</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Виталий</t>
+          <t>Григорий</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Валерьевич</t>
+          <t>Васильевич</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>vitalii17@bk.ru</t>
+          <t>grishamerzlikin@gmail.com</t>
         </is>
       </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t>Трекинг, измерение энергии и получение диагностических изображений с использованием кремниевых пиксельных сенсоров</t>
+          <t>Реконструкция трёхмерного дозового рапсределения при облучении биологических объектов пучками протонов высокой интенсивности</t>
         </is>
       </c>
     </row>
     <row r="174" ht="159.6" customHeight="1">
       <c r="A174" t="inlineStr">
         <is>
-          <t>S7-06</t>
+          <t>S7-07</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -12269,21 +12493,21 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Мерзликин</t>
+          <t>Яковлев</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Григорий</t>
+          <t>Иван</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Васильевич</t>
+          <t>Андреевич</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -12293,19 +12517,19 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>grishamerzlikin@gmail.com</t>
+          <t>iv.a.yakovlev@gmail.com</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>Реконструкция трёхмерного дозового рапсределения при облучении биологических объектов пучками протонов высокой интенсивности</t>
+          <t>Расчет характеристик черенковского детектора для контроля пучков протонов, используемых для флэш-терапии</t>
         </is>
       </c>
     </row>
     <row r="175" ht="290.1" customHeight="1">
       <c r="A175" t="inlineStr">
         <is>
-          <t>S7-07</t>
+          <t>S7-08</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -12314,43 +12538,43 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Яковлев</t>
+          <t>Зябченков</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Иван</t>
+          <t>Владислав</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Андреевич</t>
+          <t>Олегович</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>iv.a.yakovlev@gmail.com</t>
+          <t>vladislavzyabchenkov@mail.ru</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>Расчет характеристик черенковского детектора для контроля пучков протонов, используемых для флэш-терапии</t>
+          <t>Количественная оценка содержания тория и урана в свинце для радиационной защиты методом ИСП-МС</t>
         </is>
       </c>
     </row>
     <row r="176" ht="231.95" customHeight="1">
       <c r="A176" t="inlineStr">
         <is>
-          <t>S7-08</t>
+          <t>S7-09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -12359,43 +12583,43 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Зябченков</t>
+          <t>Копылова</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Владислав</t>
+          <t>Екатерина</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Олегович</t>
+          <t>Александровна</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>vladislavzyabchenkov@mail.ru</t>
+          <t>ekaterinakalip@gmail.com</t>
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>Количественная оценка содержания тория и урана в свинце для радиационной защиты методом ИСП-МС</t>
+          <t>Применение деформируемой регистрации изображений в лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="177" ht="217.5" customHeight="1">
       <c r="A177" t="inlineStr">
         <is>
-          <t>S7-09</t>
+          <t>S7-10</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -12404,43 +12628,38 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Копылова</t>
+          <t>Мамаева</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Екатерина</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>Александровна</t>
+          <t>Саргылана</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СФВУ (Якутия)</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>ekaterinakalip@gmail.com</t>
+          <t>sargylana_mamaeva@mail.ru</t>
         </is>
       </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>Применение деформируемой регистрации изображений в лучевой терапии</t>
+          <t>Биофизическая модель электрических характеристик эритроцитов при лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="178" ht="174" customHeight="1">
       <c r="A178" t="inlineStr">
         <is>
-          <t>S7-10</t>
+          <t>S7-11</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -12449,38 +12668,43 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Мамаева</t>
+          <t>Мерзликин</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Саргылана</t>
+          <t>Григорий</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Васильевич</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>СФВУ (Якутия)</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>sargylana_mamaeva@mail.ru</t>
+          <t>grishamerzlikin@gmail.com</t>
         </is>
       </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t>Биофизическая модель электрических характеристик эритроцитов при лучевой терапии</t>
+          <t>Корректировка и валидация алгоритма оценки прбега протонов в различных матералах на основании КТ-исследований</t>
         </is>
       </c>
     </row>
     <row r="179" ht="318.95" customHeight="1">
       <c r="A179" t="inlineStr">
         <is>
-          <t>S7-11</t>
+          <t>S7-12</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -12489,43 +12713,43 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Мерзликин</t>
+          <t>Ашрапов</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Григорий</t>
+          <t>Улугбек</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Васильевич</t>
+          <t>Товфикович</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>INR Uzbekistan</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>grishamerzlikin@gmail.com</t>
+          <t>ashrapov@inp.uz</t>
         </is>
       </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t>Корректировка и валидация алгоритма оценки прбега протонов в различных матералах на основании КТ-исследований</t>
+          <t>Использование гамма-облученного оксида алюминия для изготовления генераторов технеция-99М</t>
         </is>
       </c>
     </row>
     <row r="180" ht="318.95" customHeight="1">
       <c r="A180" t="inlineStr">
         <is>
-          <t>S7-12</t>
+          <t>S7-13</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -12534,43 +12758,38 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Ашрапов</t>
+          <t>Кузьменков</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Улугбек</t>
+          <t>Антон</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Товфикович</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>INR Uzbekistan</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>ashrapov@inp.uz</t>
+          <t>zhelton@yandex.ru</t>
         </is>
       </c>
       <c r="I180" s="4" t="inlineStr">
         <is>
-          <t>Использование гамма-облученного оксида алюминия для изготовления генераторов технеция-99М</t>
+          <t>Фотоядерное получение медицинских изотопов рения на осмиевых и иридиевых мишенях</t>
         </is>
       </c>
     </row>
     <row r="181" ht="231.95" customHeight="1">
       <c r="A181" t="inlineStr">
         <is>
-          <t>S7-13</t>
+          <t>S7-14</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -12579,38 +12798,38 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Кузьменков</t>
+          <t>Yusupov</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Антон</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>Александрович</t>
+          <t>Mirjalol</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>zhelton@yandex.ru</t>
+          <t>ymirjalol@bk.ru</t>
         </is>
       </c>
       <c r="I181" s="4" t="inlineStr">
         <is>
-          <t>Фотоядерное получение медицинских изотопов рения на осмиевых и иридиевых мишенях</t>
+          <t>Ядерные реакции на кислороде, углероде, азоте и боре при облучении протонным пучком 160 МэВ</t>
         </is>
       </c>
     </row>
     <row r="182" ht="217.5" customHeight="1">
       <c r="A182" t="inlineStr">
         <is>
-          <t>S7-14</t>
+          <t>S7-15</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -12619,38 +12838,43 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Yusupov</t>
+          <t>Пятаев</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Mirjalol</t>
+          <t>Дмитрий</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>МКНЦ, МГУ</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>ymirjalol@bk.ru</t>
+          <t>pataevdima2@gmail.com</t>
         </is>
       </c>
       <c r="I182" s="4" t="inlineStr">
         <is>
-          <t>Ядерные реакции на кислороде, углероде, азоте и боре при облучении протонным пучком 160 МэВ</t>
+          <t>Исследование влияния термопластических масок на поверхностную дозу и дозовое распределение в лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="183" ht="159.6" customHeight="1">
       <c r="A183" t="inlineStr">
         <is>
-          <t>S7-15</t>
+          <t>S7-16</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -12659,43 +12883,43 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Пятаев</t>
+          <t>Оганян</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Дмитрий</t>
+          <t>Ваге</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Николаевич</t>
+          <t>Робертович</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>МКНЦ, МГУ</t>
+          <t>МИФИ, МКНЦ</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>pataevdima2@gmail.com</t>
+          <t>vahe.ohanyan2000@yandex.ru</t>
         </is>
       </c>
       <c r="I183" s="4" t="inlineStr">
         <is>
-          <t>Исследование влияния термопластических масок на поверхностную дозу и дозовое распределение в лучевой терапии</t>
+          <t>Биофизическое моделирование распределения температуры при гипертермии: обзор алгоритмов и проектирование расчётного модуля.</t>
         </is>
       </c>
     </row>
     <row r="184" ht="174" customHeight="1">
       <c r="A184" t="inlineStr">
         <is>
-          <t>S7-16</t>
+          <t>S7-17</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -12704,43 +12928,43 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Оганян</t>
+          <t>Онищук</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Ваге</t>
+          <t>Елена</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Робертович</t>
+          <t>Александровна</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>МИФИ, МКНЦ</t>
+          <t>ИАЭ Обнинск</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>vahe.ohanyan2000@yandex.ru</t>
+          <t>elenaonischuk@yandex.ru</t>
         </is>
       </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t>Биофизическое моделирование распределения температуры при гипертермии: обзор алгоритмов и проектирование расчётного модуля.</t>
+          <t>Optimization of photoneutron source parameters for boron neutron capture therapy</t>
         </is>
       </c>
     </row>
     <row r="185" ht="275.45" customHeight="1">
       <c r="A185" t="inlineStr">
         <is>
-          <t>S7-17</t>
+          <t>S7-18</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -12749,43 +12973,43 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Онищук</t>
+          <t>Балачков</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Елена</t>
+          <t>Максим</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Александровна</t>
+          <t>Михайлович</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>ИАЭ Обнинск</t>
+          <t>ТПУ (Томск)</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>elenaonischuk@yandex.ru</t>
+          <t>mmb2@tpu.ru</t>
         </is>
       </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>Optimization of photoneutron source parameters for boron neutron capture therapy</t>
+          <t>Спектральные измерения пучка быстрых нейтронов циклотрона У-120</t>
         </is>
       </c>
     </row>
     <row r="186" ht="203.1" customHeight="1">
       <c r="A186" t="inlineStr">
         <is>
-          <t>S7-18</t>
+          <t>S7-19</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -12794,43 +13018,43 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Балачков</t>
+          <t>Сабуров</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Максим</t>
+          <t>Вячеслав</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Михайлович</t>
+          <t>Олегович</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>ТПУ (Томск)</t>
+          <t>МРНЦ им. А.Ф. Цыба</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>mmb2@tpu.ru</t>
+          <t>vosaburov@gmail.com</t>
         </is>
       </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>Спектральные измерения пучка быстрых нейтронов циклотрона У-120</t>
+          <t>Статус проекта по созданию комплекса нейтронной терапии на базе компактного нейтронного генератора НГ-24МТ</t>
         </is>
       </c>
     </row>
     <row r="187" ht="217.5" customHeight="1">
       <c r="A187" t="inlineStr">
         <is>
-          <t>S7-19</t>
+          <t>S7-20</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -12839,21 +13063,21 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Сабуров</t>
+          <t>Соловьев</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Вячеслав</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Олегович</t>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -12863,19 +13087,19 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>vosaburov@gmail.com</t>
+          <t>salonf@mrrc.obninsk.ru</t>
         </is>
       </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>Статус проекта по созданию комплекса нейтронной терапии на базе компактного нейтронного генератора НГ-24МТ</t>
+          <t>Особенности вычислительного прогнозирования отклика ионизационных камер для радиотерапевтического применения</t>
         </is>
       </c>
     </row>
     <row r="188" ht="231.95" customHeight="1">
       <c r="A188" t="inlineStr">
         <is>
-          <t>S7-20</t>
+          <t>S7-21</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -12884,43 +13108,43 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Соловьев</t>
+          <t>Хуцистова</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Алана</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Николаевич</t>
+          <t>Отариевна</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>МРНЦ им. А.Ф. Цыба</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>salonf@mrrc.obninsk.ru</t>
+          <t>www.alanakhutS1@mail.ru</t>
         </is>
       </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>Особенности вычислительного прогнозирования отклика ионизационных камер для радиотерапевтического применения</t>
+          <t>Моделирование комбинированного воздействия ионизирующего излучения и озона для стерилизации биоматериалов</t>
         </is>
       </c>
     </row>
     <row r="189" ht="246.6" customHeight="1">
       <c r="A189" t="inlineStr">
         <is>
-          <t>S7-21</t>
+          <t>S7-22</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -12929,21 +13153,21 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Хуцистова</t>
+          <t>Запорожская</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Алана</t>
+          <t>Ксения</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Отариевна</t>
+          <t>Васильевна</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -12953,19 +13177,19 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>www.alanakhutS1@mail.ru</t>
+          <t>zaporozhskayakv@my.msu.ru</t>
         </is>
       </c>
       <c r="I189" s="4" t="inlineStr">
         <is>
-          <t>Моделирование комбинированного воздействия ионизирующего излучения и озона для стерилизации биоматериалов</t>
+          <t>Применение шумоподавляющих фильтров при плёночной дозиметрии радиохирургических планов лечения</t>
         </is>
       </c>
     </row>
     <row r="190" ht="304.5" customHeight="1">
       <c r="A190" t="inlineStr">
         <is>
-          <t>S7-22</t>
+          <t>S7-23</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -12974,21 +13198,21 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Запорожская</t>
+          <t>Новикова</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Ксения</t>
+          <t>Евгения</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Васильевна</t>
+          <t>Антоновна</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -12998,19 +13222,19 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>zaporozhskayakv@my.msu.ru</t>
+          <t>evgeniyanovikovazar@gmail.com</t>
         </is>
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>Применение шумоподавляющих фильтров при плёночной дозиметрии радиохирургических планов лечения</t>
+          <t>Методика дозиметрии источника для электронной поверхностной брахитерапии</t>
         </is>
       </c>
     </row>
     <row r="191" ht="159.6" customHeight="1">
       <c r="A191" t="inlineStr">
         <is>
-          <t>S7-23</t>
+          <t>S7-24</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -13019,84 +13243,40 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Новикова</t>
+          <t>Петрова</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Евгения</t>
+          <t>Кристина</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Антоновна</t>
+          <t>Алексеевна</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СФВУ (Якутия)</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>evgeniyanovikovazar@gmail.com</t>
+          <t>kristinan_1604@mail.ru</t>
         </is>
       </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>Методика дозиметрии источника для электронной поверхностной брахитерапии</t>
-        </is>
-      </c>
-    </row>
-    <row r="192" ht="174" customHeight="1">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>S7-24</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C192" t="n">
-        <v>24</v>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>Петрова</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Кристина</t>
-        </is>
-      </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>Алексеевна</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>СФВУ (Якутия)</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>kristinan_1604@mail.ru</t>
-        </is>
-      </c>
-      <c r="I192" s="4" t="inlineStr">
-        <is>
           <t>Накопление золошлаковых отходов и выбросов котельного комплекса и рост онкологической заболеваемости</t>
         </is>
       </c>
     </row>
+    <row r="192" ht="174" customHeight="1"/>
     <row r="193" ht="261" customHeight="1"/>
     <row r="194" ht="261" customHeight="1"/>
     <row r="195" ht="290.1" customHeight="1"/>
@@ -13119,7 +13299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14845,6 +15025,48 @@
       <c r="H48" t="inlineStr">
         <is>
           <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>POST-48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Мальцев</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Николай</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Александрович</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>СПбГУ</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>n.maltsev@spbu.ru</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Особенности изучения свойств пучков тяжёлых ионов высоких энергий</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -14864,7 +15086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14948,6 +15170,21 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>46283.86111111111</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Председатели секционных заседаний. Доклад Н. А. Мальцева перенесён в постерную сессию. Время постеров 23.09, 16:45–18:00.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Section session chairs published. N. A. Maltsev’s talk moved to the poster session. Poster session time 23 Sep, 16:45–18:00.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update programme data and regenerate site data.js. Reorder Izosimov's two talks, swap another two talks, update affiliation
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -96,6 +96,9 @@
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3270,8 +3273,6 @@
           <t>холл2</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -5643,10 +5644,8 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="C20" t="n">
+        <v>31</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -6438,10 +6437,8 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="C36" t="n">
+        <v>14</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -8031,7 +8028,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -8164,10 +8161,8 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="C75" t="n">
+        <v>8</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -10927,7 +10922,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>НИЦ КИ-ПИЯФ</t>
+          <t>НИЦ КИ-ПИЯФ, СПбПУ</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -15086,7 +15081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15185,6 +15180,21 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>46286.56041666667</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Перестановки докладов: И. Н. Изосимов (секция 2) и Е. А. Шевчик поменялись местами во вторник; пленарные М. И. Шитова и А. Ефимова — среда и суббота. Организация Д. А. Иванищева: НИЦ КИ-ПИЯФ, СПбПУ.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Talks swapped: I. N. Izosimov (section 2) and E. A. Shevchik on Tuesday; plenaries of M. I. Shitov and A. Efimov — Wednesday and Saturday. Affiliation of D. A. Ivanishchev: NRC KI–PNPI, SPbPU.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update .gitignore to include new image file for slot machine; enhance README.md with warnings for overlapping talk schedules; improve print styles in app.css for better presentation of cancelled talks; ; increment versioning in index.html and related files for cache management consistency.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -1301,6 +1301,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1761,6 +1766,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -2130,6 +2140,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2499,6 +2514,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2873,6 +2893,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3242,6 +3267,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3452,6 +3482,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3872,6 +3907,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -4241,6 +4281,11 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -4541,6 +4586,11 @@
       <c r="F83" t="inlineStr">
         <is>
           <t>Coffee break</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>235ц</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update programme data for NUCLEUS-2026 conference, including new session details and event timings; increment versioning in data.js, index.html, and sw.js for cache management consistency.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -20,13 +20,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="170" formatCode="HH:MM"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -79,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -99,6 +100,7 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1022,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2456,7 +2458,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>0.65625</v>
+        <v>0.6354166666666666</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2470,7 +2472,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>8-14</t>
+          <t>8,10-13</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2651,7 +2653,7 @@
         <v>0.6770833333333334</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.75</v>
+        <v>0.6979166666666666</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2665,7 +2667,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>15-21</t>
+          <t>18-19</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3209,7 +3211,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.65625</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3223,7 +3225,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1-8</t>
+          <t>1-7</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4201,7 +4203,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>117л</t>
+          <t>315л</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -4295,7 +4297,7 @@
         <v>0.6770833333333334</v>
       </c>
       <c r="C77" s="3" t="n">
-        <v>0.75</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -4309,12 +4311,12 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>22-27</t>
+          <t>22-26</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>117л</t>
+          <t>315л</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4377,7 +4379,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C79" s="3" t="n">
-        <v>0.6145833333333334</v>
+        <v>0.65625</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -4391,12 +4393,12 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>22-24</t>
+          <t>22-28</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>315л</t>
+          <t>117л</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4622,6 +4624,47 @@
       <c r="I84" t="inlineStr">
         <is>
           <t>235ц</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B85" s="11" t="n">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="C85" s="11" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>секция</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>29-32</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>С. Мамаева</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>S. Mamaeva</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S191"/>
+  <dimension ref="A1:S190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10321,11 +10364,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -11919,7 +11962,7 @@
     <row r="160" ht="130.5" customHeight="1">
       <c r="A160" t="inlineStr">
         <is>
-          <t>S6-01</t>
+          <t>S6-02</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -11932,39 +11975,39 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Дербин</t>
+          <t>Кондратьев</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Александр</t>
+          <t>Владимир</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Владимирович</t>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>ПИЯФ</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>derbin_av@pnpi.nrcki.ru</t>
+          <t>vkondrat@theor.jinr.ru</t>
         </is>
       </c>
       <c r="I160" s="4" t="inlineStr">
         <is>
-          <t>Поиск тяжелого стерильного нейтрино в бета-распаде ¹⁴⁴Pr</t>
+          <t>Эффекты динамо и осцилляций в спектрах нейтрино сверхновых</t>
         </is>
       </c>
     </row>
     <row r="161" ht="246.6" customHeight="1">
       <c r="A161" t="inlineStr">
         <is>
-          <t>S6-02</t>
+          <t>S6-03</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -12002,14 +12045,14 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>Эффекты динамо и осцилляций в спектрах нейтрино сверхновых</t>
+          <t>Эффекты намагниченности ядер во взрывном нуклеосинтезе</t>
         </is>
       </c>
     </row>
     <row r="162" ht="231.95" customHeight="1">
       <c r="A162" t="inlineStr">
         <is>
-          <t>S6-03</t>
+          <t>S6-04</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -12022,17 +12065,12 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Кондратьев</t>
+          <t>Лубашевский</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Владимир</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>Николаевич</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -12042,19 +12080,19 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>vkondrat@theor.jinr.ru</t>
+          <t>lubashev@jinr.ru</t>
         </is>
       </c>
       <c r="I162" s="4" t="inlineStr">
         <is>
-          <t>Эффекты намагниченности ядер во взрывном нуклеосинтезе</t>
+          <t>Search for rare processes within the νGeN experiment at Kalinin nuclear power plant</t>
         </is>
       </c>
     </row>
     <row r="163" ht="57.95" customHeight="1">
       <c r="A163" t="inlineStr">
         <is>
-          <t>S6-04</t>
+          <t>S6-05</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -12067,34 +12105,39 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Лубашевский</t>
+          <t>Громов</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Максим</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Борисович</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>НИИЯФ</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>lubashev@jinr.ru</t>
+          <t>gromov@physics.msu.ru</t>
         </is>
       </c>
       <c r="I163" s="4" t="inlineStr">
         <is>
-          <t>Search for rare processes within the νGeN experiment at Kalinin nuclear power plant</t>
+          <t>Precise reactor antineutrino spectrum measurement with TAO detector</t>
         </is>
       </c>
     </row>
     <row r="164" ht="130.5" customHeight="1">
       <c r="A164" t="inlineStr">
         <is>
-          <t>S6-05</t>
+          <t>S6-06</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -12107,17 +12150,17 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Громов</t>
+          <t>Михеев</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Максим</t>
+          <t>Семён</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Борисович</t>
+          <t>Алексеевич</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -12127,19 +12170,19 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>gromov@physics.msu.ru</t>
+          <t>semenmihey@gmail.com</t>
         </is>
       </c>
       <c r="I164" s="4" t="inlineStr">
         <is>
-          <t>Precise reactor antineutrino spectrum measurement with TAO detector</t>
+          <t>Условия появления Λ-гиперонов в материи нейтронных звёзд в моделях среднего поля</t>
         </is>
       </c>
     </row>
     <row r="165" ht="101.45" customHeight="1">
       <c r="A165" t="inlineStr">
         <is>
-          <t>S6-06</t>
+          <t>S6-07</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -12152,39 +12195,34 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Михеев</t>
+          <t>Kabir</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Семён</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>Алексеевич</t>
+          <t>Abdul</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>НИИЯФ</t>
+          <t>Institute of Space Technology (Islamabad, Pakistan)</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>semenmihey@gmail.com</t>
+          <t>kabirkhanak1@gmail.com</t>
         </is>
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>Условия появления Λ-гиперонов в материи нейтронных звёзд в моделях среднего поля</t>
+          <t>Analysis of radiative capture of proton ¹¹B (p, γ) ¹²C at low energy</t>
         </is>
       </c>
     </row>
     <row r="166" ht="217.5" customHeight="1">
       <c r="A166" t="inlineStr">
         <is>
-          <t>S6-07</t>
+          <t>S6-08</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -12197,74 +12235,74 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Kabir</t>
+          <t>Le</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Abdul</t>
+          <t>Huy Viet</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Institute of Space Technology (Islamabad, Pakistan)</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>kabirkhanak1@gmail.com</t>
+          <t>leviethuy1@duytan.edu.vn</t>
         </is>
       </c>
       <c r="I166" s="4" t="inlineStr">
         <is>
-          <t>Analysis of radiative capture of proton ¹¹B (p, γ) ¹²C at low energy</t>
+          <t>Characterization of the cosmic muon background in the νGeN experiment</t>
         </is>
       </c>
     </row>
     <row r="167" ht="144.95" customHeight="1">
       <c r="A167" t="inlineStr">
         <is>
-          <t>S6-08</t>
+          <t>S7-01</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Le</t>
+          <t>Киселев</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Huy Viet</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>ОИЯИ</t>
+          <t>Василий</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Алексеевич</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>leviethuy1@duytan.edu.vn</t>
+          <t>kiselevva@fnkcrio.ru</t>
         </is>
       </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>Characterization of the cosmic muon background in the νGeN experiment</t>
+          <t>Подход к оптимизации распределения поглощенной дозы в биологическом объекте в лучевой терапии пучком ускоренных протонов</t>
         </is>
       </c>
     </row>
     <row r="168" ht="174" customHeight="1">
       <c r="A168" t="inlineStr">
         <is>
-          <t>S7-01</t>
+          <t>S7-02</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -12273,38 +12311,43 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Киселев</t>
+          <t>Щербаков</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Василий</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Алексеевич</t>
+          <t>Александрович</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>kiselevva@fnkcrio.ru</t>
+          <t>sherbakov.aa15@physics.msu.ru</t>
         </is>
       </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>Подход к оптимизации распределения поглощенной дозы в биологическом объекте в лучевой терапии пучком ускоренных протонов</t>
+          <t>Оценка рисков развития радиационно-индуцированных заболеваний при проведении лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="169" ht="144.95" customHeight="1">
       <c r="A169" t="inlineStr">
         <is>
-          <t>S7-02</t>
+          <t>S7-03</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -12313,43 +12356,43 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Щербаков</t>
+          <t>Васильева</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Алина</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Александрович</t>
+          <t>Геннадиевна</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>НИЦ КИ ИФВЭ</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>sherbakov.aa15@physics.msu.ru</t>
+          <t>vasilyeva-ag@ihep.ru</t>
         </is>
       </c>
       <c r="I169" s="4" t="inlineStr">
         <is>
-          <t>Оценка рисков развития радиационно-индуцированных заболеваний при проведении лучевой терапии</t>
+          <t>Измерение сечения реакции ¹²C(¹²C,X)¹¹C: особенности эксперимента и оценка неопределенностей</t>
         </is>
       </c>
     </row>
     <row r="170" ht="188.45" customHeight="1">
       <c r="A170" t="inlineStr">
         <is>
-          <t>S7-03</t>
+          <t>S7-04</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -12358,21 +12401,21 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Васильева</t>
+          <t>Парменова</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Алина</t>
+          <t>Екатерина</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Геннадиевна</t>
+          <t>Владимировна</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -12382,19 +12425,19 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>vasilyeva-ag@ihep.ru</t>
+          <t>Ekaterina.Parmenova@ihep.ru</t>
         </is>
       </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t>Измерение сечения реакции ¹²C(¹²C,X)¹¹C: особенности эксперимента и оценка неопределенностей</t>
+          <t>Реализация работы с данными КТ в системе планирования ионной лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="171" ht="159.6" customHeight="1">
       <c r="A171" t="inlineStr">
         <is>
-          <t>S7-04</t>
+          <t>S7-05</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -12403,43 +12446,43 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Парменова</t>
+          <t>Петров</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Екатерина</t>
+          <t>Виталий</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Владимировна</t>
+          <t>Валерьевич</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>НИЦ КИ ИФВЭ</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Ekaterina.Parmenova@ihep.ru</t>
+          <t>vitalii17@bk.ru</t>
         </is>
       </c>
       <c r="I171" s="4" t="inlineStr">
         <is>
-          <t>Реализация работы с данными КТ в системе планирования ионной лучевой терапии</t>
+          <t>Трекинг, измерение энергии и получение диагностических изображений с использованием кремниевых пиксельных сенсоров</t>
         </is>
       </c>
     </row>
     <row r="172" ht="203.1" customHeight="1">
       <c r="A172" t="inlineStr">
         <is>
-          <t>S7-05</t>
+          <t>S7-06</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -12448,43 +12491,43 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Петров</t>
+          <t>Мерзликин</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Виталий</t>
+          <t>Григорий</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Валерьевич</t>
+          <t>Васильевич</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>СПбГУ</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>vitalii17@bk.ru</t>
+          <t>grishamerzlikin@gmail.com</t>
         </is>
       </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>Трекинг, измерение энергии и получение диагностических изображений с использованием кремниевых пиксельных сенсоров</t>
+          <t>Реконструкция трёхмерного дозового рапсределения при облучении биологических объектов пучками протонов высокой интенсивности</t>
         </is>
       </c>
     </row>
     <row r="173" ht="159.6" customHeight="1">
       <c r="A173" t="inlineStr">
         <is>
-          <t>S7-06</t>
+          <t>S7-07</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -12493,21 +12536,21 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Мерзликин</t>
+          <t>Яковлев</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Григорий</t>
+          <t>Иван</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Васильевич</t>
+          <t>Андреевич</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -12517,19 +12560,19 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>grishamerzlikin@gmail.com</t>
+          <t>iv.a.yakovlev@gmail.com</t>
         </is>
       </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t>Реконструкция трёхмерного дозового рапсределения при облучении биологических объектов пучками протонов высокой интенсивности</t>
+          <t>Расчет характеристик черенковского детектора для контроля пучков протонов, используемых для флэш-терапии</t>
         </is>
       </c>
     </row>
     <row r="174" ht="159.6" customHeight="1">
       <c r="A174" t="inlineStr">
         <is>
-          <t>S7-07</t>
+          <t>S7-08</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -12538,43 +12581,43 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Яковлев</t>
+          <t>Зябченков</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Иван</t>
+          <t>Владислав</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Андреевич</t>
+          <t>Олегович</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>ОИЯИ</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>iv.a.yakovlev@gmail.com</t>
+          <t>vladislavzyabchenkov@mail.ru</t>
         </is>
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>Расчет характеристик черенковского детектора для контроля пучков протонов, используемых для флэш-терапии</t>
+          <t>Количественная оценка содержания тория и урана в свинце для радиационной защиты методом ИСП-МС</t>
         </is>
       </c>
     </row>
     <row r="175" ht="290.1" customHeight="1">
       <c r="A175" t="inlineStr">
         <is>
-          <t>S7-08</t>
+          <t>S7-09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -12583,43 +12626,43 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Зябченков</t>
+          <t>Копылова</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Владислав</t>
+          <t>Екатерина</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Олегович</t>
+          <t>Александровна</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>ОИЯИ</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>vladislavzyabchenkov@mail.ru</t>
+          <t>ekaterinakalip@gmail.com</t>
         </is>
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>Количественная оценка содержания тория и урана в свинце для радиационной защиты методом ИСП-МС</t>
+          <t>Применение деформируемой регистрации изображений в лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="176" ht="231.95" customHeight="1">
       <c r="A176" t="inlineStr">
         <is>
-          <t>S7-09</t>
+          <t>S7-10</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -12628,43 +12671,38 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Копылова</t>
+          <t>Мамаева</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Екатерина</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>Александровна</t>
+          <t>Саргылана</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СФВУ (Якутия)</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>ekaterinakalip@gmail.com</t>
+          <t>sargylana_mamaeva@mail.ru</t>
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>Применение деформируемой регистрации изображений в лучевой терапии</t>
+          <t>Биофизическая модель электрических характеристик эритроцитов при лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="177" ht="217.5" customHeight="1">
       <c r="A177" t="inlineStr">
         <is>
-          <t>S7-10</t>
+          <t>S7-11</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -12673,38 +12711,43 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Мамаева</t>
+          <t>Мерзликин</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Саргылана</t>
+          <t>Григорий</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Васильевич</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>СФВУ (Якутия)</t>
+          <t>ИЯИ РАН</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>sargylana_mamaeva@mail.ru</t>
+          <t>grishamerzlikin@gmail.com</t>
         </is>
       </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>Биофизическая модель электрических характеристик эритроцитов при лучевой терапии</t>
+          <t>Корректировка и валидация алгоритма оценки прбега протонов в различных матералах на основании КТ-исследований</t>
         </is>
       </c>
     </row>
     <row r="178" ht="174" customHeight="1">
       <c r="A178" t="inlineStr">
         <is>
-          <t>S7-11</t>
+          <t>S7-12</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -12713,43 +12756,43 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Мерзликин</t>
+          <t>Ашрапов</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Григорий</t>
+          <t>Улугбек</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Васильевич</t>
+          <t>Товфикович</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>ИЯИ РАН</t>
+          <t>INR Uzbekistan</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>grishamerzlikin@gmail.com</t>
+          <t>ashrapov@inp.uz</t>
         </is>
       </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t>Корректировка и валидация алгоритма оценки прбега протонов в различных матералах на основании КТ-исследований</t>
+          <t>Использование гамма-облученного оксида алюминия для изготовления генераторов технеция-99М</t>
         </is>
       </c>
     </row>
     <row r="179" ht="318.95" customHeight="1">
       <c r="A179" t="inlineStr">
         <is>
-          <t>S7-12</t>
+          <t>S7-13</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -12758,43 +12801,38 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Ашрапов</t>
+          <t>Кузьменков</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Улугбек</t>
+          <t>Антон</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Товфикович</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>INR Uzbekistan</t>
+          <t>Александрович</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ashrapov@inp.uz</t>
+          <t>zhelton@yandex.ru</t>
         </is>
       </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t>Использование гамма-облученного оксида алюминия для изготовления генераторов технеция-99М</t>
+          <t>Фотоядерное получение медицинских изотопов рения на осмиевых и иридиевых мишенях</t>
         </is>
       </c>
     </row>
     <row r="180" ht="318.95" customHeight="1">
       <c r="A180" t="inlineStr">
         <is>
-          <t>S7-13</t>
+          <t>S7-14</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -12803,38 +12841,38 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Кузьменков</t>
+          <t>Yusupov</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Антон</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>Александрович</t>
+          <t>Mirjalol</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>zhelton@yandex.ru</t>
+          <t>ymirjalol@bk.ru</t>
         </is>
       </c>
       <c r="I180" s="4" t="inlineStr">
         <is>
-          <t>Фотоядерное получение медицинских изотопов рения на осмиевых и иридиевых мишенях</t>
+          <t>Ядерные реакции на кислороде, углероде, азоте и боре при облучении протонным пучком 160 МэВ</t>
         </is>
       </c>
     </row>
     <row r="181" ht="231.95" customHeight="1">
       <c r="A181" t="inlineStr">
         <is>
-          <t>S7-14</t>
+          <t>S7-15</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -12843,38 +12881,43 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Yusupov</t>
+          <t>Пятаев</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Mirjalol</t>
+          <t>Дмитрий</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>МКНЦ, МГУ</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>ymirjalol@bk.ru</t>
+          <t>pataevdima2@gmail.com</t>
         </is>
       </c>
       <c r="I181" s="4" t="inlineStr">
         <is>
-          <t>Ядерные реакции на кислороде, углероде, азоте и боре при облучении протонным пучком 160 МэВ</t>
+          <t>Исследование влияния термопластических масок на поверхностную дозу и дозовое распределение в лучевой терапии</t>
         </is>
       </c>
     </row>
     <row r="182" ht="217.5" customHeight="1">
       <c r="A182" t="inlineStr">
         <is>
-          <t>S7-15</t>
+          <t>S7-16</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -12883,43 +12926,43 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Пятаев</t>
+          <t>Оганян</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Дмитрий</t>
+          <t>Ваге</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Николаевич</t>
+          <t>Робертович</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>МКНЦ, МГУ</t>
+          <t>МИФИ, МКНЦ</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>pataevdima2@gmail.com</t>
+          <t>vahe.ohanyan2000@yandex.ru</t>
         </is>
       </c>
       <c r="I182" s="4" t="inlineStr">
         <is>
-          <t>Исследование влияния термопластических масок на поверхностную дозу и дозовое распределение в лучевой терапии</t>
+          <t>Биофизическое моделирование распределения температуры при гипертермии: обзор алгоритмов и проектирование расчётного модуля.</t>
         </is>
       </c>
     </row>
     <row r="183" ht="159.6" customHeight="1">
       <c r="A183" t="inlineStr">
         <is>
-          <t>S7-16</t>
+          <t>S7-17</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -12928,43 +12971,43 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Оганян</t>
+          <t>Онищук</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Ваге</t>
+          <t>Елена</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Робертович</t>
+          <t>Александровна</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>МИФИ, МКНЦ</t>
+          <t>ИАЭ Обнинск</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>vahe.ohanyan2000@yandex.ru</t>
+          <t>elenaonischuk@yandex.ru</t>
         </is>
       </c>
       <c r="I183" s="4" t="inlineStr">
         <is>
-          <t>Биофизическое моделирование распределения температуры при гипертермии: обзор алгоритмов и проектирование расчётного модуля.</t>
+          <t>Optimization of photoneutron source parameters for boron neutron capture therapy</t>
         </is>
       </c>
     </row>
     <row r="184" ht="174" customHeight="1">
       <c r="A184" t="inlineStr">
         <is>
-          <t>S7-17</t>
+          <t>S7-18</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -12973,43 +13016,43 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Онищук</t>
+          <t>Балачков</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Елена</t>
+          <t>Максим</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Александровна</t>
+          <t>Михайлович</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>ИАЭ Обнинск</t>
+          <t>ТПУ (Томск)</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>elenaonischuk@yandex.ru</t>
+          <t>mmb2@tpu.ru</t>
         </is>
       </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t>Optimization of photoneutron source parameters for boron neutron capture therapy</t>
+          <t>Спектральные измерения пучка быстрых нейтронов циклотрона У-120</t>
         </is>
       </c>
     </row>
     <row r="185" ht="275.45" customHeight="1">
       <c r="A185" t="inlineStr">
         <is>
-          <t>S7-18</t>
+          <t>S7-19</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -13018,43 +13061,43 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Балачков</t>
+          <t>Сабуров</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Максим</t>
+          <t>Вячеслав</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Михайлович</t>
+          <t>Олегович</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>ТПУ (Томск)</t>
+          <t>МРНЦ им. А.Ф. Цыба</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>mmb2@tpu.ru</t>
+          <t>vosaburov@gmail.com</t>
         </is>
       </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>Спектральные измерения пучка быстрых нейтронов циклотрона У-120</t>
+          <t>Статус проекта по созданию комплекса нейтронной терапии на базе компактного нейтронного генератора НГ-24МТ</t>
         </is>
       </c>
     </row>
     <row r="186" ht="203.1" customHeight="1">
       <c r="A186" t="inlineStr">
         <is>
-          <t>S7-19</t>
+          <t>S7-20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -13063,21 +13106,21 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Сабуров</t>
+          <t>Соловьев</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Вячеслав</t>
+          <t>Алексей</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Олегович</t>
+          <t>Николаевич</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -13087,19 +13130,19 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>vosaburov@gmail.com</t>
+          <t>salonf@mrrc.obninsk.ru</t>
         </is>
       </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>Статус проекта по созданию комплекса нейтронной терапии на базе компактного нейтронного генератора НГ-24МТ</t>
+          <t>Особенности вычислительного прогнозирования отклика ионизационных камер для радиотерапевтического применения</t>
         </is>
       </c>
     </row>
     <row r="187" ht="217.5" customHeight="1">
       <c r="A187" t="inlineStr">
         <is>
-          <t>S7-20</t>
+          <t>S7-21</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -13108,43 +13151,43 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Соловьев</t>
+          <t>Хуцистова</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Алексей</t>
+          <t>Алана</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Николаевич</t>
+          <t>Отариевна</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>МРНЦ им. А.Ф. Цыба</t>
+          <t>МГУ</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>salonf@mrrc.obninsk.ru</t>
+          <t>www.alanakhutS1@mail.ru</t>
         </is>
       </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>Особенности вычислительного прогнозирования отклика ионизационных камер для радиотерапевтического применения</t>
+          <t>Моделирование комбинированного воздействия ионизирующего излучения и озона для стерилизации биоматериалов</t>
         </is>
       </c>
     </row>
     <row r="188" ht="231.95" customHeight="1">
       <c r="A188" t="inlineStr">
         <is>
-          <t>S7-21</t>
+          <t>S7-22</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -13153,21 +13196,21 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Хуцистова</t>
+          <t>Запорожская</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Алана</t>
+          <t>Ксения</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Отариевна</t>
+          <t>Васильевна</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -13177,19 +13220,19 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>www.alanakhutS1@mail.ru</t>
+          <t>zaporozhskayakv@my.msu.ru</t>
         </is>
       </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>Моделирование комбинированного воздействия ионизирующего излучения и озона для стерилизации биоматериалов</t>
+          <t>Применение шумоподавляющих фильтров при плёночной дозиметрии радиохирургических планов лечения</t>
         </is>
       </c>
     </row>
     <row r="189" ht="246.6" customHeight="1">
       <c r="A189" t="inlineStr">
         <is>
-          <t>S7-22</t>
+          <t>S7-23</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -13198,21 +13241,21 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Запорожская</t>
+          <t>Новикова</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Ксения</t>
+          <t>Евгения</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Васильевна</t>
+          <t>Антоновна</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -13222,19 +13265,19 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>zaporozhskayakv@my.msu.ru</t>
+          <t>evgeniyanovikovazar@gmail.com</t>
         </is>
       </c>
       <c r="I189" s="4" t="inlineStr">
         <is>
-          <t>Применение шумоподавляющих фильтров при плёночной дозиметрии радиохирургических планов лечения</t>
+          <t>Методика дозиметрии источника для электронной поверхностной брахитерапии</t>
         </is>
       </c>
     </row>
     <row r="190" ht="304.5" customHeight="1">
       <c r="A190" t="inlineStr">
         <is>
-          <t>S7-23</t>
+          <t>S7-24</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -13243,84 +13286,40 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Новикова</t>
+          <t>Петрова</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Евгения</t>
+          <t>Кристина</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Антоновна</t>
+          <t>Алексеевна</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>МГУ</t>
+          <t>СФВУ (Якутия)</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>evgeniyanovikovazar@gmail.com</t>
+          <t>kristinan_1604@mail.ru</t>
         </is>
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>Методика дозиметрии источника для электронной поверхностной брахитерапии</t>
-        </is>
-      </c>
-    </row>
-    <row r="191" ht="159.6" customHeight="1">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>S7-24</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C191" t="n">
-        <v>24</v>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>Петрова</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Кристина</t>
-        </is>
-      </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>Алексеевна</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>СФВУ (Якутия)</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>kristinan_1604@mail.ru</t>
-        </is>
-      </c>
-      <c r="I191" s="4" t="inlineStr">
-        <is>
           <t>Накопление золошлаковых отходов и выбросов котельного комплекса и рост онкологической заболеваемости</t>
         </is>
       </c>
     </row>
+    <row r="191" ht="159.6" customHeight="1"/>
     <row r="192" ht="174" customHeight="1"/>
     <row r="193" ht="261" customHeight="1"/>
     <row r="194" ht="261" customHeight="1"/>
@@ -15131,7 +15130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15245,6 +15244,51 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>46287.68680555555</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>А. В. Дербин не приедет: его доклад снят, секция 6 в среду начинается в 14:00 без него. В пятницу секция 3 — в 315л, секция 7 — в 117л.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>A. V. Derbin will not attend: his talk is removed, and section 6 on Wednesday starts at 14:00 without it. On Friday, section 3 is in 315л and section 7 is in 117л.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>46287.71666666667</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Секция 7: Е. А. Копылова, M. Yusupov, Д. Н. Пятаев и В. Р. Оганян перенесены на пятницу, 14:45–15:45, после уже стоящих докладов. Остальные доклады секции 7 во вторник сдвинуты вперёд.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Section 7: E. A. Kopylova, M. Yusupov, D. N. Pyataev and V. R. Ohanyan are moved to Friday 14:45–15:45, after the existing section 7 talks. The other Tuesday section 7 talks move up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>46287.73333333333</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Секция 7 в пятницу после кофе, 16:15–17:15, 117л: А. С. Петровская, затем Е. А. Онищук, А. Н. Соловьев и А. О. Хуцистова. Вечерняя секция 7 во вторник сокращена.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Section 7 on Friday after coffee, 16:15–17:15, room 117л: A. S. Petrovskaya, then E. A. Onishchuk, A. N. Solovyev and A. O. Khutsistova. Tuesday evening section 7 is shortened.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update programme data for NUCLEUS-2026 conference, including new session details and event timings; increment versioning in data.js, index.html, and sw.js for cache management consistency; update stylesheet and script references in index.html for cache-busting.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -20,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
@@ -28,6 +28,7 @@
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="170" formatCode="HH:MM"/>
+    <numFmt numFmtId="171" formatCode="DD.MM.YYYY HH:MM"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -80,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,6 +102,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15130,7 +15132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15289,6 +15291,21 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>46287.83541666667</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>В «Сетке» выделите день и нажмите «Подробный день»: время, аудитории и председатели заседаний. Печать этого дня — один альбомный лист A4.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>In Overview, highlight a day and press Detailed day for times, rooms, and sitting chairs. Print that day as one landscape A4.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Boat excursion rescheduled, site rebuilt
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -3676,10 +3676,10 @@
         <v>46289</v>
       </c>
       <c r="B62" s="3" t="n">
-        <v>0.625</v>
+        <v>0.6458333333333334</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>0.7291666666666666</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -15132,7 +15132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15306,6 +15306,21 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>46288.56111111111</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Экскурсия на теплоходе в четверг перенесена на 15:30–18:30.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Thursday boat excursion moved to 15:30–18:30.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>